<commit_message>
Update `cpi_u_rs` with row for 2024
</commit_message>
<xml_diff>
--- a/data-raw/cpi_u_rs.xlsx
+++ b/data-raw/cpi_u_rs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Akin_B\OneDrive - US Department of Labor - BLS\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\March 2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5B199323-DD2D-4274-B22D-14FCF0F50907}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCD3BFA0-4106-4EDE-85AC-1E3C92BA40FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="All items" sheetId="1" r:id="rId1"/>
@@ -64,6 +64,12 @@
     <t>AVG</t>
   </si>
   <si>
+    <t>Consumer Price Index Retroactive Series (R-CPI-U-RS)</t>
+  </si>
+  <si>
+    <t>U.S. city average</t>
+  </si>
+  <si>
     <t>All items</t>
   </si>
   <si>
@@ -71,12 +77,6 @@
   </si>
   <si>
     <t>December 1977=100</t>
-  </si>
-  <si>
-    <t>U.S. city average</t>
-  </si>
-  <si>
-    <t>Consumer Price Index Retroactive Series (R-CPI-U-RS)</t>
   </si>
 </sst>
 </file>
@@ -86,7 +86,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -98,24 +98,19 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -142,38 +137,38 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -479,2198 +474,2268 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O53"/>
+  <dimension ref="A1:O54"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.33203125" customWidth="1"/>
-    <col min="2" max="14" width="6.77734375" customWidth="1"/>
-    <col min="15" max="15" width="47.77734375" customWidth="1"/>
+    <col min="1" max="1" width="6.88671875" customWidth="1"/>
+    <col min="2" max="6" width="5.77734375" customWidth="1"/>
+    <col min="7" max="7" width="6.88671875" customWidth="1"/>
+    <col min="8" max="8" width="5.77734375" customWidth="1"/>
+    <col min="9" max="9" width="6.88671875" customWidth="1"/>
+    <col min="10" max="13" width="5.77734375" customWidth="1"/>
+    <col min="14" max="14" width="5.5546875" customWidth="1"/>
+    <col min="15" max="15" width="51.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="10"/>
+      <c r="J1" s="10"/>
+      <c r="K1" s="10"/>
+      <c r="L1" s="10"/>
+      <c r="M1" s="10"/>
+      <c r="N1" s="10"/>
+      <c r="O1" s="10"/>
+    </row>
+    <row r="2" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="10"/>
+      <c r="I2" s="10"/>
+      <c r="J2" s="10"/>
+      <c r="K2" s="10"/>
+      <c r="L2" s="10"/>
+      <c r="M2" s="10"/>
+      <c r="N2" s="10"/>
+      <c r="O2" s="10"/>
+    </row>
+    <row r="3" spans="1:15" s="10" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="10"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="10"/>
+      <c r="E4" s="10"/>
+      <c r="F4" s="10"/>
+      <c r="G4" s="10"/>
+      <c r="H4" s="10"/>
+      <c r="I4" s="10"/>
+      <c r="J4" s="10"/>
+      <c r="K4" s="10"/>
+      <c r="L4" s="10"/>
+      <c r="M4" s="10"/>
+      <c r="N4" s="10"/>
+      <c r="O4" s="10"/>
+    </row>
+    <row r="5" spans="1:15" s="10" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
-      <c r="N1" s="4"/>
-      <c r="O1" s="4"/>
-    </row>
-    <row r="2" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
-      <c r="L2" s="4"/>
-      <c r="M2" s="4"/>
-      <c r="N2" s="4"/>
-      <c r="O2" s="4"/>
-    </row>
-    <row r="3" spans="1:15" s="4" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4"/>
-      <c r="K4" s="4"/>
-      <c r="L4" s="4"/>
-      <c r="M4" s="4"/>
-      <c r="N4" s="4"/>
-      <c r="O4" s="4"/>
-    </row>
-    <row r="5" spans="1:15" s="4" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="8" t="s">
+    </row>
+    <row r="6" spans="1:15" s="9" customFormat="1" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="F6" s="9" t="s">
+      <c r="F6" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G6" s="9" t="s">
+      <c r="G6" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="H6" s="9" t="s">
+      <c r="H6" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="I6" s="9" t="s">
+      <c r="I6" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="J6" s="9" t="s">
+      <c r="J6" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="K6" s="9" t="s">
+      <c r="K6" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="L6" s="9" t="s">
+      <c r="L6" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="M6" s="9" t="s">
+      <c r="M6" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="N6" s="10" t="s">
+      <c r="N6" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="O6" s="1"/>
-    </row>
-    <row r="7" spans="1:15" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="2">
+      <c r="O6" s="8"/>
+    </row>
+    <row r="7" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="3">
         <v>1977</v>
       </c>
-      <c r="B7" s="11"/>
-      <c r="C7" s="11"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11"/>
-      <c r="G7" s="11"/>
-      <c r="H7" s="11"/>
-      <c r="I7" s="11"/>
-      <c r="J7" s="11"/>
-      <c r="K7" s="11"/>
-      <c r="L7" s="11"/>
-      <c r="M7" s="3">
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+      <c r="G7" s="4"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="4"/>
+      <c r="J7" s="4"/>
+      <c r="K7" s="4"/>
+      <c r="L7" s="4"/>
+      <c r="M7" s="5">
         <v>100</v>
       </c>
-      <c r="N7" s="11"/>
-      <c r="O7" s="1"/>
-    </row>
-    <row r="8" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="2">
+      <c r="N7" s="4"/>
+      <c r="O7" s="2"/>
+    </row>
+    <row r="8" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="3">
         <v>1978</v>
       </c>
-      <c r="B8" s="3">
+      <c r="B8" s="5">
         <v>100.5</v>
       </c>
-      <c r="C8" s="3">
+      <c r="C8" s="5">
         <v>101.1</v>
       </c>
-      <c r="D8" s="3">
+      <c r="D8" s="5">
         <v>101.8</v>
       </c>
-      <c r="E8" s="3">
+      <c r="E8" s="5">
         <v>102.7</v>
       </c>
-      <c r="F8" s="3">
+      <c r="F8" s="5">
         <v>103.6</v>
       </c>
-      <c r="G8" s="3">
+      <c r="G8" s="5">
         <v>104.5</v>
       </c>
-      <c r="H8" s="3">
+      <c r="H8" s="5">
         <v>105</v>
       </c>
-      <c r="I8" s="3">
+      <c r="I8" s="5">
         <v>105.5</v>
       </c>
-      <c r="J8" s="3">
+      <c r="J8" s="5">
         <v>106.1</v>
       </c>
-      <c r="K8" s="3">
+      <c r="K8" s="5">
         <v>106.7</v>
       </c>
-      <c r="L8" s="3">
+      <c r="L8" s="5">
         <v>107.3</v>
       </c>
-      <c r="M8" s="3">
+      <c r="M8" s="5">
         <v>107.8</v>
       </c>
-      <c r="N8" s="3">
+      <c r="N8" s="5">
         <v>104.4</v>
       </c>
-      <c r="O8" s="1"/>
-    </row>
-    <row r="9" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="2">
+      <c r="O8" s="2"/>
+    </row>
+    <row r="9" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="3">
         <v>1979</v>
       </c>
-      <c r="B9" s="3">
+      <c r="B9" s="5">
         <v>108.7</v>
       </c>
-      <c r="C9" s="3">
+      <c r="C9" s="5">
         <v>109.7</v>
       </c>
-      <c r="D9" s="3">
+      <c r="D9" s="5">
         <v>110.7</v>
       </c>
-      <c r="E9" s="3">
+      <c r="E9" s="5">
         <v>111.8</v>
       </c>
-      <c r="F9" s="3">
+      <c r="F9" s="5">
         <v>113</v>
       </c>
-      <c r="G9" s="3">
+      <c r="G9" s="5">
         <v>114.1</v>
       </c>
-      <c r="H9" s="3">
+      <c r="H9" s="5">
         <v>115.1</v>
       </c>
-      <c r="I9" s="3">
+      <c r="I9" s="5">
         <v>116</v>
       </c>
-      <c r="J9" s="3">
+      <c r="J9" s="5">
         <v>117.1</v>
       </c>
-      <c r="K9" s="3">
+      <c r="K9" s="5">
         <v>117.9</v>
       </c>
-      <c r="L9" s="3">
+      <c r="L9" s="5">
         <v>118.5</v>
       </c>
-      <c r="M9" s="3">
+      <c r="M9" s="5">
         <v>119.5</v>
       </c>
-      <c r="N9" s="3">
+      <c r="N9" s="5">
         <v>114.3</v>
       </c>
-      <c r="O9" s="1"/>
-    </row>
-    <row r="10" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="2">
+      <c r="O9" s="2"/>
+    </row>
+    <row r="10" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="3">
         <v>1980</v>
       </c>
-      <c r="B10" s="3">
+      <c r="B10" s="5">
         <v>120.8</v>
       </c>
-      <c r="C10" s="3">
+      <c r="C10" s="5">
         <v>122.4</v>
       </c>
-      <c r="D10" s="3">
+      <c r="D10" s="5">
         <v>123.8</v>
       </c>
-      <c r="E10" s="3">
+      <c r="E10" s="5">
         <v>124.7</v>
       </c>
-      <c r="F10" s="3">
+      <c r="F10" s="5">
         <v>125.7</v>
       </c>
-      <c r="G10" s="3">
+      <c r="G10" s="5">
         <v>126.7</v>
       </c>
-      <c r="H10" s="3">
+      <c r="H10" s="5">
         <v>127.5</v>
       </c>
-      <c r="I10" s="3">
+      <c r="I10" s="5">
         <v>128.6</v>
       </c>
-      <c r="J10" s="3">
+      <c r="J10" s="5">
         <v>129.9</v>
       </c>
-      <c r="K10" s="3">
+      <c r="K10" s="5">
         <v>130.69999999999999</v>
       </c>
-      <c r="L10" s="3">
+      <c r="L10" s="5">
         <v>131.5</v>
       </c>
-      <c r="M10" s="3">
+      <c r="M10" s="5">
         <v>132.4</v>
       </c>
-      <c r="N10" s="3">
+      <c r="N10" s="5">
         <v>127.1</v>
       </c>
-      <c r="O10" s="1"/>
-    </row>
-    <row r="11" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="2">
+      <c r="O10" s="2"/>
+    </row>
+    <row r="11" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="3">
         <v>1981</v>
       </c>
-      <c r="B11" s="3">
+      <c r="B11" s="5">
         <v>133.6</v>
       </c>
-      <c r="C11" s="3">
+      <c r="C11" s="5">
         <v>135.19999999999999</v>
       </c>
-      <c r="D11" s="3">
+      <c r="D11" s="5">
         <v>136.30000000000001</v>
       </c>
-      <c r="E11" s="3">
+      <c r="E11" s="5">
         <v>137.1</v>
       </c>
-      <c r="F11" s="3">
+      <c r="F11" s="5">
         <v>137.9</v>
       </c>
-      <c r="G11" s="3">
+      <c r="G11" s="5">
         <v>138.69999999999999</v>
       </c>
-      <c r="H11" s="3">
+      <c r="H11" s="5">
         <v>139.69999999999999</v>
       </c>
-      <c r="I11" s="3">
+      <c r="I11" s="5">
         <v>140.69999999999999</v>
       </c>
-      <c r="J11" s="3">
+      <c r="J11" s="5">
         <v>141.80000000000001</v>
       </c>
-      <c r="K11" s="3">
+      <c r="K11" s="5">
         <v>142.4</v>
       </c>
-      <c r="L11" s="3">
+      <c r="L11" s="5">
         <v>142.9</v>
       </c>
-      <c r="M11" s="3">
+      <c r="M11" s="5">
         <v>143.4</v>
       </c>
-      <c r="N11" s="3">
+      <c r="N11" s="5">
         <v>139.1</v>
       </c>
-      <c r="O11" s="1"/>
-    </row>
-    <row r="12" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="2">
+      <c r="O11" s="2"/>
+    </row>
+    <row r="12" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="3">
         <v>1982</v>
       </c>
-      <c r="B12" s="3">
+      <c r="B12" s="5">
         <v>144.19999999999999</v>
       </c>
-      <c r="C12" s="3">
+      <c r="C12" s="5">
         <v>144.69999999999999</v>
       </c>
-      <c r="D12" s="3">
+      <c r="D12" s="5">
         <v>144.9</v>
       </c>
-      <c r="E12" s="3">
+      <c r="E12" s="5">
         <v>145</v>
       </c>
-      <c r="F12" s="3">
+      <c r="F12" s="5">
         <v>146.1</v>
       </c>
-      <c r="G12" s="3">
+      <c r="G12" s="5">
         <v>147.5</v>
       </c>
-      <c r="H12" s="3">
+      <c r="H12" s="5">
         <v>148.5</v>
       </c>
-      <c r="I12" s="3">
+      <c r="I12" s="5">
         <v>148.80000000000001</v>
       </c>
-      <c r="J12" s="3">
+      <c r="J12" s="5">
         <v>149.5</v>
       </c>
-      <c r="K12" s="3">
+      <c r="K12" s="5">
         <v>150.19999999999999</v>
       </c>
-      <c r="L12" s="3">
+      <c r="L12" s="5">
         <v>150.5</v>
       </c>
-      <c r="M12" s="3">
+      <c r="M12" s="5">
         <v>150.6</v>
       </c>
-      <c r="N12" s="3">
+      <c r="N12" s="5">
         <v>147.5</v>
       </c>
-      <c r="O12" s="1"/>
-    </row>
-    <row r="13" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="2">
+      <c r="O12" s="2"/>
+    </row>
+    <row r="13" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="3">
         <v>1983</v>
       </c>
-      <c r="B13" s="3">
+      <c r="B13" s="5">
         <v>151</v>
       </c>
-      <c r="C13" s="3">
+      <c r="C13" s="5">
         <v>151.1</v>
       </c>
-      <c r="D13" s="3">
+      <c r="D13" s="5">
         <v>151.19999999999999</v>
       </c>
-      <c r="E13" s="3">
+      <c r="E13" s="5">
         <v>152.4</v>
       </c>
-      <c r="F13" s="3">
+      <c r="F13" s="5">
         <v>153.19999999999999</v>
       </c>
-      <c r="G13" s="3">
+      <c r="G13" s="5">
         <v>153.69999999999999</v>
       </c>
-      <c r="H13" s="3">
+      <c r="H13" s="5">
         <v>154.30000000000001</v>
       </c>
-      <c r="I13" s="3">
+      <c r="I13" s="5">
         <v>154.80000000000001</v>
       </c>
-      <c r="J13" s="3">
+      <c r="J13" s="5">
         <v>155.6</v>
       </c>
-      <c r="K13" s="3">
+      <c r="K13" s="5">
         <v>156</v>
       </c>
-      <c r="L13" s="3">
+      <c r="L13" s="5">
         <v>156.1</v>
       </c>
-      <c r="M13" s="3">
+      <c r="M13" s="5">
         <v>156.30000000000001</v>
       </c>
-      <c r="N13" s="3">
+      <c r="N13" s="5">
         <v>153.80000000000001</v>
       </c>
-      <c r="O13" s="1"/>
-    </row>
-    <row r="14" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="2">
+      <c r="O13" s="2"/>
+    </row>
+    <row r="14" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="3">
         <v>1984</v>
       </c>
-      <c r="B14" s="3">
+      <c r="B14" s="5">
         <v>157.19999999999999</v>
       </c>
-      <c r="C14" s="3">
+      <c r="C14" s="5">
         <v>158</v>
       </c>
-      <c r="D14" s="3">
+      <c r="D14" s="5">
         <v>158.30000000000001</v>
       </c>
-      <c r="E14" s="3">
+      <c r="E14" s="5">
         <v>159</v>
       </c>
-      <c r="F14" s="3">
+      <c r="F14" s="5">
         <v>159.5</v>
       </c>
-      <c r="G14" s="3">
+      <c r="G14" s="5">
         <v>159.9</v>
       </c>
-      <c r="H14" s="3">
+      <c r="H14" s="5">
         <v>160.4</v>
       </c>
-      <c r="I14" s="3">
+      <c r="I14" s="5">
         <v>161.1</v>
       </c>
-      <c r="J14" s="3">
+      <c r="J14" s="5">
         <v>161.80000000000001</v>
       </c>
-      <c r="K14" s="3">
+      <c r="K14" s="5">
         <v>162.19999999999999</v>
       </c>
-      <c r="L14" s="3">
+      <c r="L14" s="5">
         <v>162.19999999999999</v>
       </c>
-      <c r="M14" s="3">
+      <c r="M14" s="5">
         <v>162.30000000000001</v>
       </c>
-      <c r="N14" s="3">
+      <c r="N14" s="5">
         <v>160.19999999999999</v>
       </c>
-      <c r="O14" s="1"/>
-    </row>
-    <row r="15" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="2">
+      <c r="O14" s="2"/>
+    </row>
+    <row r="15" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="3">
         <v>1985</v>
       </c>
-      <c r="B15" s="3">
+      <c r="B15" s="5">
         <v>162.5</v>
       </c>
-      <c r="C15" s="3">
+      <c r="C15" s="5">
         <v>163.19999999999999</v>
       </c>
-      <c r="D15" s="3">
+      <c r="D15" s="5">
         <v>163.9</v>
       </c>
-      <c r="E15" s="3">
+      <c r="E15" s="5">
         <v>164.6</v>
       </c>
-      <c r="F15" s="3">
+      <c r="F15" s="5">
         <v>165.2</v>
       </c>
-      <c r="G15" s="3">
+      <c r="G15" s="5">
         <v>165.6</v>
       </c>
-      <c r="H15" s="3">
+      <c r="H15" s="5">
         <v>165.9</v>
       </c>
-      <c r="I15" s="3">
+      <c r="I15" s="5">
         <v>166.2</v>
       </c>
-      <c r="J15" s="3">
+      <c r="J15" s="5">
         <v>166.8</v>
       </c>
-      <c r="K15" s="3">
+      <c r="K15" s="5">
         <v>167.2</v>
       </c>
-      <c r="L15" s="3">
+      <c r="L15" s="5">
         <v>167.7</v>
       </c>
-      <c r="M15" s="3">
+      <c r="M15" s="5">
         <v>168.1</v>
       </c>
-      <c r="N15" s="3">
+      <c r="N15" s="5">
         <v>165.6</v>
       </c>
-      <c r="O15" s="1"/>
-    </row>
-    <row r="16" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="2">
+      <c r="O15" s="2"/>
+    </row>
+    <row r="16" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="3">
         <v>1986</v>
       </c>
-      <c r="B16" s="3">
+      <c r="B16" s="5">
         <v>168.6</v>
       </c>
-      <c r="C16" s="3">
+      <c r="C16" s="5">
         <v>168.1</v>
       </c>
-      <c r="D16" s="3">
+      <c r="D16" s="5">
         <v>167.3</v>
       </c>
-      <c r="E16" s="3">
+      <c r="E16" s="5">
         <v>166.9</v>
       </c>
-      <c r="F16" s="3">
+      <c r="F16" s="5">
         <v>167.4</v>
       </c>
-      <c r="G16" s="3">
+      <c r="G16" s="5">
         <v>168.2</v>
       </c>
-      <c r="H16" s="3">
+      <c r="H16" s="5">
         <v>168.2</v>
       </c>
-      <c r="I16" s="3">
+      <c r="I16" s="5">
         <v>168.5</v>
       </c>
-      <c r="J16" s="3">
+      <c r="J16" s="5">
         <v>169.4</v>
       </c>
-      <c r="K16" s="3">
+      <c r="K16" s="5">
         <v>169.5</v>
       </c>
-      <c r="L16" s="3">
+      <c r="L16" s="5">
         <v>169.5</v>
       </c>
-      <c r="M16" s="3">
+      <c r="M16" s="5">
         <v>169.6</v>
       </c>
-      <c r="N16" s="3">
+      <c r="N16" s="5">
         <v>168.4</v>
       </c>
-      <c r="O16" s="1"/>
-    </row>
-    <row r="17" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="2">
+      <c r="O16" s="2"/>
+    </row>
+    <row r="17" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="3">
         <v>1987</v>
       </c>
-      <c r="B17" s="3">
+      <c r="B17" s="5">
         <v>170.6</v>
       </c>
-      <c r="C17" s="3">
+      <c r="C17" s="5">
         <v>171.3</v>
       </c>
-      <c r="D17" s="3">
+      <c r="D17" s="5">
         <v>172</v>
       </c>
-      <c r="E17" s="3">
+      <c r="E17" s="5">
         <v>172.9</v>
       </c>
-      <c r="F17" s="3">
+      <c r="F17" s="5">
         <v>173.4</v>
       </c>
-      <c r="G17" s="3">
+      <c r="G17" s="5">
         <v>174</v>
       </c>
-      <c r="H17" s="3">
+      <c r="H17" s="5">
         <v>174.3</v>
       </c>
-      <c r="I17" s="3">
+      <c r="I17" s="5">
         <v>175.3</v>
       </c>
-      <c r="J17" s="3">
+      <c r="J17" s="5">
         <v>176.1</v>
       </c>
-      <c r="K17" s="3">
+      <c r="K17" s="5">
         <v>176.5</v>
       </c>
-      <c r="L17" s="3">
+      <c r="L17" s="5">
         <v>176.6</v>
       </c>
-      <c r="M17" s="3">
+      <c r="M17" s="5">
         <v>176.5</v>
       </c>
-      <c r="N17" s="3">
+      <c r="N17" s="5">
         <v>174.1</v>
       </c>
-      <c r="O17" s="1"/>
-    </row>
-    <row r="18" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="2">
+      <c r="O17" s="2"/>
+    </row>
+    <row r="18" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="3">
         <v>1988</v>
       </c>
-      <c r="B18" s="3">
+      <c r="B18" s="5">
         <v>177</v>
       </c>
-      <c r="C18" s="3">
+      <c r="C18" s="5">
         <v>177.3</v>
       </c>
-      <c r="D18" s="3">
+      <c r="D18" s="5">
         <v>178</v>
       </c>
-      <c r="E18" s="3">
+      <c r="E18" s="5">
         <v>178.9</v>
       </c>
-      <c r="F18" s="3">
+      <c r="F18" s="5">
         <v>179.5</v>
       </c>
-      <c r="G18" s="3">
+      <c r="G18" s="5">
         <v>180.1</v>
       </c>
-      <c r="H18" s="3">
+      <c r="H18" s="5">
         <v>180.8</v>
       </c>
-      <c r="I18" s="3">
+      <c r="I18" s="5">
         <v>181.6</v>
       </c>
-      <c r="J18" s="3">
+      <c r="J18" s="5">
         <v>182.7</v>
       </c>
-      <c r="K18" s="3">
+      <c r="K18" s="5">
         <v>183.2</v>
       </c>
-      <c r="L18" s="3">
+      <c r="L18" s="5">
         <v>183.3</v>
       </c>
-      <c r="M18" s="3">
+      <c r="M18" s="5">
         <v>183.4</v>
       </c>
-      <c r="N18" s="3">
+      <c r="N18" s="5">
         <v>180.5</v>
       </c>
-      <c r="O18" s="1"/>
-    </row>
-    <row r="19" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="2">
+      <c r="O18" s="2"/>
+    </row>
+    <row r="19" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="3">
         <v>1989</v>
       </c>
-      <c r="B19" s="3">
+      <c r="B19" s="5">
         <v>184.3</v>
       </c>
-      <c r="C19" s="3">
+      <c r="C19" s="5">
         <v>184.9</v>
       </c>
-      <c r="D19" s="3">
+      <c r="D19" s="5">
         <v>185.9</v>
       </c>
-      <c r="E19" s="3">
+      <c r="E19" s="5">
         <v>187.2</v>
       </c>
-      <c r="F19" s="3">
+      <c r="F19" s="5">
         <v>188.1</v>
       </c>
-      <c r="G19" s="3">
+      <c r="G19" s="5">
         <v>188.5</v>
       </c>
-      <c r="H19" s="3">
+      <c r="H19" s="5">
         <v>189</v>
       </c>
-      <c r="I19" s="3">
+      <c r="I19" s="5">
         <v>189.2</v>
       </c>
-      <c r="J19" s="3">
+      <c r="J19" s="5">
         <v>189.8</v>
       </c>
-      <c r="K19" s="3">
+      <c r="K19" s="5">
         <v>190.6</v>
       </c>
-      <c r="L19" s="3">
+      <c r="L19" s="5">
         <v>190.9</v>
       </c>
-      <c r="M19" s="3">
+      <c r="M19" s="5">
         <v>191.1</v>
       </c>
-      <c r="N19" s="3">
+      <c r="N19" s="5">
         <v>188.3</v>
       </c>
-      <c r="O19" s="1"/>
-    </row>
-    <row r="20" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="2">
+      <c r="O19" s="2"/>
+    </row>
+    <row r="20" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="3">
         <v>1990</v>
       </c>
-      <c r="B20" s="3">
+      <c r="B20" s="5">
         <v>193</v>
       </c>
-      <c r="C20" s="3">
+      <c r="C20" s="5">
         <v>193.9</v>
       </c>
-      <c r="D20" s="3">
+      <c r="D20" s="5">
         <v>194.9</v>
       </c>
-      <c r="E20" s="3">
+      <c r="E20" s="5">
         <v>195.2</v>
       </c>
-      <c r="F20" s="3">
+      <c r="F20" s="5">
         <v>195.5</v>
       </c>
-      <c r="G20" s="3">
+      <c r="G20" s="5">
         <v>196.5</v>
       </c>
-      <c r="H20" s="3">
+      <c r="H20" s="5">
         <v>197.3</v>
       </c>
-      <c r="I20" s="3">
+      <c r="I20" s="5">
         <v>199</v>
       </c>
-      <c r="J20" s="3">
+      <c r="J20" s="5">
         <v>200.6</v>
       </c>
-      <c r="K20" s="3">
+      <c r="K20" s="5">
         <v>201.7</v>
       </c>
-      <c r="L20" s="3">
+      <c r="L20" s="5">
         <v>202</v>
       </c>
-      <c r="M20" s="3">
+      <c r="M20" s="5">
         <v>202</v>
       </c>
-      <c r="N20" s="3">
+      <c r="N20" s="5">
         <v>197.6</v>
       </c>
-      <c r="O20" s="1"/>
-    </row>
-    <row r="21" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="2">
+      <c r="O20" s="2"/>
+    </row>
+    <row r="21" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3">
         <v>1991</v>
       </c>
-      <c r="B21" s="3">
+      <c r="B21" s="5">
         <v>202.9</v>
       </c>
-      <c r="C21" s="3">
+      <c r="C21" s="5">
         <v>203.1</v>
       </c>
-      <c r="D21" s="3">
+      <c r="D21" s="5">
         <v>203.3</v>
       </c>
-      <c r="E21" s="3">
+      <c r="E21" s="5">
         <v>203.5</v>
       </c>
-      <c r="F21" s="3">
+      <c r="F21" s="5">
         <v>204.1</v>
       </c>
-      <c r="G21" s="3">
+      <c r="G21" s="5">
         <v>204.5</v>
       </c>
-      <c r="H21" s="3">
+      <c r="H21" s="5">
         <v>204.7</v>
       </c>
-      <c r="I21" s="3">
+      <c r="I21" s="5">
         <v>205.2</v>
       </c>
-      <c r="J21" s="3">
+      <c r="J21" s="5">
         <v>206.1</v>
       </c>
-      <c r="K21" s="3">
+      <c r="K21" s="5">
         <v>206.2</v>
       </c>
-      <c r="L21" s="3">
+      <c r="L21" s="5">
         <v>206.7</v>
       </c>
-      <c r="M21" s="3">
+      <c r="M21" s="5">
         <v>206.8</v>
       </c>
-      <c r="N21" s="3">
+      <c r="N21" s="5">
         <v>204.8</v>
       </c>
-      <c r="O21" s="1"/>
-    </row>
-    <row r="22" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="2">
+      <c r="O21" s="2"/>
+    </row>
+    <row r="22" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3">
         <v>1992</v>
       </c>
-      <c r="B22" s="3">
+      <c r="B22" s="5">
         <v>207.2</v>
       </c>
-      <c r="C22" s="3">
+      <c r="C22" s="5">
         <v>207.7</v>
       </c>
-      <c r="D22" s="3">
+      <c r="D22" s="5">
         <v>208.6</v>
       </c>
-      <c r="E22" s="3">
+      <c r="E22" s="5">
         <v>209</v>
       </c>
-      <c r="F22" s="3">
+      <c r="F22" s="5">
         <v>209.3</v>
       </c>
-      <c r="G22" s="3">
+      <c r="G22" s="5">
         <v>209.7</v>
       </c>
-      <c r="H22" s="3">
+      <c r="H22" s="5">
         <v>210.1</v>
       </c>
-      <c r="I22" s="3">
+      <c r="I22" s="5">
         <v>210.6</v>
       </c>
-      <c r="J22" s="3">
+      <c r="J22" s="5">
         <v>211.2</v>
       </c>
-      <c r="K22" s="3">
+      <c r="K22" s="5">
         <v>211.8</v>
       </c>
-      <c r="L22" s="3">
+      <c r="L22" s="5">
         <v>212.1</v>
       </c>
-      <c r="M22" s="3">
+      <c r="M22" s="5">
         <v>211.9</v>
       </c>
-      <c r="N22" s="3">
+      <c r="N22" s="5">
         <v>209.9</v>
       </c>
-      <c r="O22" s="1"/>
-    </row>
-    <row r="23" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="2">
+      <c r="O22" s="2"/>
+    </row>
+    <row r="23" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3">
         <v>1993</v>
       </c>
-      <c r="B23" s="3">
+      <c r="B23" s="5">
         <v>212.6</v>
       </c>
-      <c r="C23" s="3">
+      <c r="C23" s="5">
         <v>213.3</v>
       </c>
-      <c r="D23" s="3">
+      <c r="D23" s="5">
         <v>214</v>
       </c>
-      <c r="E23" s="3">
+      <c r="E23" s="5">
         <v>214.5</v>
       </c>
-      <c r="F23" s="3">
+      <c r="F23" s="5">
         <v>215</v>
       </c>
-      <c r="G23" s="3">
+      <c r="G23" s="5">
         <v>215.2</v>
       </c>
-      <c r="H23" s="3">
+      <c r="H23" s="5">
         <v>215.3</v>
       </c>
-      <c r="I23" s="3">
+      <c r="I23" s="5">
         <v>215.7</v>
       </c>
-      <c r="J23" s="3">
+      <c r="J23" s="5">
         <v>216</v>
       </c>
-      <c r="K23" s="3">
+      <c r="K23" s="5">
         <v>216.7</v>
       </c>
-      <c r="L23" s="3">
+      <c r="L23" s="5">
         <v>216.9</v>
       </c>
-      <c r="M23" s="3">
+      <c r="M23" s="5">
         <v>216.7</v>
       </c>
-      <c r="N23" s="3">
+      <c r="N23" s="5">
         <v>215.2</v>
       </c>
-      <c r="O23" s="1"/>
-    </row>
-    <row r="24" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="2">
+      <c r="O23" s="2"/>
+    </row>
+    <row r="24" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3">
         <v>1994</v>
       </c>
-      <c r="B24" s="3">
+      <c r="B24" s="5">
         <v>217.1</v>
       </c>
-      <c r="C24" s="3">
+      <c r="C24" s="5">
         <v>217.6</v>
       </c>
-      <c r="D24" s="3">
+      <c r="D24" s="5">
         <v>218.4</v>
       </c>
-      <c r="E24" s="3">
+      <c r="E24" s="5">
         <v>218.6</v>
       </c>
-      <c r="F24" s="3">
+      <c r="F24" s="5">
         <v>218.9</v>
       </c>
-      <c r="G24" s="3">
+      <c r="G24" s="5">
         <v>219.5</v>
       </c>
-      <c r="H24" s="3">
+      <c r="H24" s="5">
         <v>220</v>
       </c>
-      <c r="I24" s="3">
+      <c r="I24" s="5">
         <v>220.7</v>
       </c>
-      <c r="J24" s="3">
+      <c r="J24" s="5">
         <v>221.1</v>
       </c>
-      <c r="K24" s="3">
+      <c r="K24" s="5">
         <v>221.2</v>
       </c>
-      <c r="L24" s="3">
+      <c r="L24" s="5">
         <v>221.5</v>
       </c>
-      <c r="M24" s="3">
+      <c r="M24" s="5">
         <v>221.4</v>
       </c>
-      <c r="N24" s="3">
+      <c r="N24" s="5">
         <v>219.7</v>
       </c>
-      <c r="O24" s="1"/>
-    </row>
-    <row r="25" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="2">
+      <c r="O24" s="2"/>
+    </row>
+    <row r="25" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3">
         <v>1995</v>
       </c>
-      <c r="B25" s="3">
+      <c r="B25" s="5">
         <v>222.2</v>
       </c>
-      <c r="C25" s="3">
+      <c r="C25" s="5">
         <v>222.9</v>
       </c>
-      <c r="D25" s="3">
+      <c r="D25" s="5">
         <v>223.6</v>
       </c>
-      <c r="E25" s="3">
+      <c r="E25" s="5">
         <v>224.3</v>
       </c>
-      <c r="F25" s="3">
+      <c r="F25" s="5">
         <v>224.7</v>
       </c>
-      <c r="G25" s="3">
+      <c r="G25" s="5">
         <v>225.2</v>
       </c>
-      <c r="H25" s="3">
+      <c r="H25" s="5">
         <v>225.3</v>
       </c>
-      <c r="I25" s="3">
+      <c r="I25" s="5">
         <v>225.7</v>
       </c>
-      <c r="J25" s="3">
+      <c r="J25" s="5">
         <v>226.1</v>
       </c>
-      <c r="K25" s="3">
+      <c r="K25" s="5">
         <v>226.7</v>
       </c>
-      <c r="L25" s="3">
+      <c r="L25" s="5">
         <v>226.5</v>
       </c>
-      <c r="M25" s="3">
+      <c r="M25" s="5">
         <v>226.4</v>
       </c>
-      <c r="N25" s="3">
+      <c r="N25" s="5">
         <v>225</v>
       </c>
-      <c r="O25" s="1"/>
-    </row>
-    <row r="26" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="2">
+      <c r="O25" s="2"/>
+    </row>
+    <row r="26" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="3">
         <v>1996</v>
       </c>
-      <c r="B26" s="3">
+      <c r="B26" s="5">
         <v>227.5</v>
       </c>
-      <c r="C26" s="3">
+      <c r="C26" s="5">
         <v>228.3</v>
       </c>
-      <c r="D26" s="3">
+      <c r="D26" s="5">
         <v>229.4</v>
       </c>
-      <c r="E26" s="3">
+      <c r="E26" s="5">
         <v>230.2</v>
       </c>
-      <c r="F26" s="3">
+      <c r="F26" s="5">
         <v>230.8</v>
       </c>
-      <c r="G26" s="3">
+      <c r="G26" s="5">
         <v>230.9</v>
       </c>
-      <c r="H26" s="3">
+      <c r="H26" s="5">
         <v>231.3</v>
       </c>
-      <c r="I26" s="3">
+      <c r="I26" s="5">
         <v>231.5</v>
       </c>
-      <c r="J26" s="3">
+      <c r="J26" s="5">
         <v>232.3</v>
       </c>
-      <c r="K26" s="3">
+      <c r="K26" s="5">
         <v>233</v>
       </c>
-      <c r="L26" s="3">
+      <c r="L26" s="5">
         <v>233.4</v>
       </c>
-      <c r="M26" s="3">
+      <c r="M26" s="5">
         <v>233.4</v>
       </c>
-      <c r="N26" s="3">
+      <c r="N26" s="5">
         <v>231</v>
       </c>
-      <c r="O26" s="1"/>
-    </row>
-    <row r="27" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="2">
+      <c r="O26" s="2"/>
+    </row>
+    <row r="27" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="3">
         <v>1997</v>
       </c>
-      <c r="B27" s="3">
+      <c r="B27" s="5">
         <v>234.1</v>
       </c>
-      <c r="C27" s="3">
+      <c r="C27" s="5">
         <v>234.7</v>
       </c>
-      <c r="D27" s="3">
+      <c r="D27" s="5">
         <v>235.2</v>
       </c>
-      <c r="E27" s="3">
+      <c r="E27" s="5">
         <v>235.5</v>
       </c>
-      <c r="F27" s="3">
+      <c r="F27" s="5">
         <v>235.4</v>
       </c>
-      <c r="G27" s="3">
+      <c r="G27" s="5">
         <v>235.8</v>
       </c>
-      <c r="H27" s="3">
+      <c r="H27" s="5">
         <v>235.9</v>
       </c>
-      <c r="I27" s="3">
+      <c r="I27" s="5">
         <v>236.3</v>
       </c>
-      <c r="J27" s="3">
+      <c r="J27" s="5">
         <v>237.1</v>
       </c>
-      <c r="K27" s="3">
+      <c r="K27" s="5">
         <v>237.5</v>
       </c>
-      <c r="L27" s="3">
+      <c r="L27" s="5">
         <v>237.4</v>
       </c>
-      <c r="M27" s="3">
+      <c r="M27" s="5">
         <v>237</v>
       </c>
-      <c r="N27" s="3">
+      <c r="N27" s="5">
         <v>236</v>
       </c>
-      <c r="O27" s="1"/>
-    </row>
-    <row r="28" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="2">
+      <c r="O27" s="2"/>
+    </row>
+    <row r="28" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="3">
         <v>1998</v>
       </c>
-      <c r="B28" s="3">
+      <c r="B28" s="5">
         <v>237.4</v>
       </c>
-      <c r="C28" s="3">
+      <c r="C28" s="5">
         <v>237.8</v>
       </c>
-      <c r="D28" s="3">
+      <c r="D28" s="5">
         <v>238.1</v>
       </c>
-      <c r="E28" s="3">
+      <c r="E28" s="5">
         <v>238.6</v>
       </c>
-      <c r="F28" s="3">
+      <c r="F28" s="5">
         <v>239</v>
       </c>
-      <c r="G28" s="3">
+      <c r="G28" s="5">
         <v>239.1</v>
       </c>
-      <c r="H28" s="3">
+      <c r="H28" s="5">
         <v>239.4</v>
       </c>
-      <c r="I28" s="3">
+      <c r="I28" s="5">
         <v>239.7</v>
       </c>
-      <c r="J28" s="3">
+      <c r="J28" s="5">
         <v>240</v>
       </c>
-      <c r="K28" s="3">
+      <c r="K28" s="5">
         <v>240.5</v>
       </c>
-      <c r="L28" s="3">
+      <c r="L28" s="5">
         <v>240.5</v>
       </c>
-      <c r="M28" s="3">
+      <c r="M28" s="5">
         <v>240.3</v>
       </c>
-      <c r="N28" s="3">
+      <c r="N28" s="5">
         <v>239.2</v>
       </c>
-      <c r="O28" s="1"/>
-    </row>
-    <row r="29" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="2">
+      <c r="O28" s="2"/>
+    </row>
+    <row r="29" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="3">
         <v>1999</v>
       </c>
-      <c r="B29" s="3">
+      <c r="B29" s="5">
         <v>240.9</v>
       </c>
-      <c r="C29" s="3">
+      <c r="C29" s="5">
         <v>241.2</v>
       </c>
-      <c r="D29" s="3">
+      <c r="D29" s="5">
         <v>241.9</v>
       </c>
-      <c r="E29" s="3">
+      <c r="E29" s="5">
         <v>243.6</v>
       </c>
-      <c r="F29" s="3">
+      <c r="F29" s="5">
         <v>243.6</v>
       </c>
-      <c r="G29" s="3">
+      <c r="G29" s="5">
         <v>243.7</v>
       </c>
-      <c r="H29" s="3">
+      <c r="H29" s="5">
         <v>244.4</v>
       </c>
-      <c r="I29" s="3">
+      <c r="I29" s="5">
         <v>245.1</v>
       </c>
-      <c r="J29" s="3">
+      <c r="J29" s="5">
         <v>246.2</v>
       </c>
-      <c r="K29" s="3">
+      <c r="K29" s="5">
         <v>246.7</v>
       </c>
-      <c r="L29" s="3">
+      <c r="L29" s="5">
         <v>246.8</v>
       </c>
-      <c r="M29" s="3">
+      <c r="M29" s="5">
         <v>246.8</v>
       </c>
-      <c r="N29" s="3">
+      <c r="N29" s="5">
         <v>244.2</v>
       </c>
-      <c r="O29" s="1"/>
-    </row>
-    <row r="30" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="2">
+      <c r="O29" s="2"/>
+    </row>
+    <row r="30" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="3">
         <v>2000</v>
       </c>
-      <c r="B30" s="3">
+      <c r="B30" s="5">
         <v>247.6</v>
       </c>
-      <c r="C30" s="3">
+      <c r="C30" s="5">
         <v>249.1</v>
       </c>
-      <c r="D30" s="3">
+      <c r="D30" s="5">
         <v>251.1</v>
       </c>
-      <c r="E30" s="3">
+      <c r="E30" s="5">
         <v>251.2</v>
       </c>
-      <c r="F30" s="3">
+      <c r="F30" s="5">
         <v>251.4</v>
       </c>
-      <c r="G30" s="3">
+      <c r="G30" s="5">
         <v>252.9</v>
       </c>
-      <c r="H30" s="3">
+      <c r="H30" s="5">
         <v>253.4</v>
       </c>
-      <c r="I30" s="3">
+      <c r="I30" s="5">
         <v>253.4</v>
       </c>
-      <c r="J30" s="3">
+      <c r="J30" s="5">
         <v>254.8</v>
       </c>
-      <c r="K30" s="3">
+      <c r="K30" s="5">
         <v>255.1</v>
       </c>
-      <c r="L30" s="3">
+      <c r="L30" s="5">
         <v>255.3</v>
       </c>
-      <c r="M30" s="3">
+      <c r="M30" s="5">
         <v>255.1</v>
       </c>
-      <c r="N30" s="3">
+      <c r="N30" s="5">
         <v>252.5</v>
       </c>
-      <c r="O30" s="1"/>
-    </row>
-    <row r="31" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="2">
+      <c r="O30" s="2"/>
+    </row>
+    <row r="31" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="3">
         <v>2001</v>
       </c>
-      <c r="B31" s="3">
+      <c r="B31" s="5">
         <v>256.8</v>
       </c>
-      <c r="C31" s="3">
+      <c r="C31" s="5">
         <v>257.89999999999998</v>
       </c>
-      <c r="D31" s="3">
+      <c r="D31" s="5">
         <v>258.5</v>
       </c>
-      <c r="E31" s="3">
+      <c r="E31" s="5">
         <v>259.5</v>
       </c>
-      <c r="F31" s="3">
+      <c r="F31" s="5">
         <v>260.5</v>
       </c>
-      <c r="G31" s="3">
+      <c r="G31" s="5">
         <v>261.10000000000002</v>
       </c>
-      <c r="H31" s="3">
+      <c r="H31" s="5">
         <v>260.3</v>
       </c>
-      <c r="I31" s="3">
+      <c r="I31" s="5">
         <v>260.39999999999998</v>
       </c>
-      <c r="J31" s="3">
+      <c r="J31" s="5">
         <v>261.39999999999998</v>
       </c>
-      <c r="K31" s="3">
+      <c r="K31" s="5">
         <v>260.60000000000002</v>
       </c>
-      <c r="L31" s="3">
+      <c r="L31" s="5">
         <v>260.10000000000002</v>
       </c>
-      <c r="M31" s="3">
+      <c r="M31" s="5">
         <v>259.10000000000002</v>
       </c>
-      <c r="N31" s="3">
+      <c r="N31" s="5">
         <v>259.7</v>
       </c>
-      <c r="O31" s="1"/>
-    </row>
-    <row r="32" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="2">
+      <c r="O31" s="2"/>
+    </row>
+    <row r="32" spans="1:15" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="3">
         <v>2002</v>
       </c>
-      <c r="B32" s="3">
+      <c r="B32" s="5">
         <v>259.8</v>
       </c>
-      <c r="C32" s="3">
+      <c r="C32" s="5">
         <v>260.8</v>
       </c>
-      <c r="D32" s="3">
+      <c r="D32" s="5">
         <v>262.2</v>
       </c>
-      <c r="E32" s="3">
+      <c r="E32" s="5">
         <v>263.7</v>
       </c>
-      <c r="F32" s="3">
+      <c r="F32" s="5">
         <v>263.60000000000002</v>
       </c>
-      <c r="G32" s="3">
+      <c r="G32" s="5">
         <v>263.89999999999998</v>
       </c>
-      <c r="H32" s="3">
+      <c r="H32" s="5">
         <v>264.10000000000002</v>
       </c>
-      <c r="I32" s="3">
+      <c r="I32" s="5">
         <v>265</v>
       </c>
-      <c r="J32" s="3">
+      <c r="J32" s="5">
         <v>265.39999999999998</v>
       </c>
-      <c r="K32" s="3">
+      <c r="K32" s="5">
         <v>265.89999999999998</v>
       </c>
-      <c r="L32" s="3">
+      <c r="L32" s="5">
         <v>265.89999999999998</v>
       </c>
-      <c r="M32" s="3">
+      <c r="M32" s="5">
         <v>265.3</v>
       </c>
-      <c r="N32" s="3">
+      <c r="N32" s="5">
         <v>263.8</v>
       </c>
       <c r="O32" s="1"/>
     </row>
-    <row r="33" spans="1:14" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="2">
+    <row r="33" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="3">
         <v>2003</v>
       </c>
-      <c r="B33" s="3">
+      <c r="B33" s="5">
         <v>266.39999999999998</v>
       </c>
-      <c r="C33" s="3">
+      <c r="C33" s="5">
         <v>268.60000000000002</v>
       </c>
-      <c r="D33" s="3">
+      <c r="D33" s="5">
         <v>270.2</v>
       </c>
-      <c r="E33" s="3">
+      <c r="E33" s="5">
         <v>269.5</v>
       </c>
-      <c r="F33" s="3">
+      <c r="F33" s="5">
         <v>269.10000000000002</v>
       </c>
-      <c r="G33" s="3">
+      <c r="G33" s="5">
         <v>269.5</v>
       </c>
-      <c r="H33" s="3">
+      <c r="H33" s="5">
         <v>269.7</v>
       </c>
-      <c r="I33" s="3">
+      <c r="I33" s="5">
         <v>270.7</v>
       </c>
-      <c r="J33" s="3">
+      <c r="J33" s="5">
         <v>271.60000000000002</v>
       </c>
-      <c r="K33" s="3">
+      <c r="K33" s="5">
         <v>271.39999999999998</v>
       </c>
-      <c r="L33" s="3">
+      <c r="L33" s="5">
         <v>270.60000000000002</v>
       </c>
-      <c r="M33" s="3">
+      <c r="M33" s="5">
         <v>270.3</v>
       </c>
-      <c r="N33" s="3">
+      <c r="N33" s="5">
         <v>269.8</v>
       </c>
-    </row>
-    <row r="34" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="2">
+      <c r="O33" s="2"/>
+    </row>
+    <row r="34" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="3">
         <v>2004</v>
       </c>
-      <c r="B34" s="3">
+      <c r="B34" s="5">
         <v>271.7</v>
       </c>
-      <c r="C34" s="3">
+      <c r="C34" s="5">
         <v>273.2</v>
       </c>
-      <c r="D34" s="3">
+      <c r="D34" s="5">
         <v>274.89999999999998</v>
       </c>
-      <c r="E34" s="3">
+      <c r="E34" s="5">
         <v>275.8</v>
       </c>
-      <c r="F34" s="3">
+      <c r="F34" s="5">
         <v>277.3</v>
       </c>
-      <c r="G34" s="3">
+      <c r="G34" s="5">
         <v>278.2</v>
       </c>
-      <c r="H34" s="3">
+      <c r="H34" s="5">
         <v>277.8</v>
       </c>
-      <c r="I34" s="3">
+      <c r="I34" s="5">
         <v>277.89999999999998</v>
       </c>
-      <c r="J34" s="3">
+      <c r="J34" s="5">
         <v>278.5</v>
       </c>
-      <c r="K34" s="3">
+      <c r="K34" s="5">
         <v>280</v>
       </c>
-      <c r="L34" s="3">
+      <c r="L34" s="5">
         <v>280.2</v>
       </c>
-      <c r="M34" s="3">
+      <c r="M34" s="5">
         <v>279.10000000000002</v>
       </c>
-      <c r="N34" s="3">
+      <c r="N34" s="5">
         <v>277</v>
       </c>
-    </row>
-    <row r="35" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="2">
+      <c r="O34" s="2"/>
+    </row>
+    <row r="35" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="3">
         <v>2005</v>
       </c>
-      <c r="B35" s="3">
+      <c r="B35" s="5">
         <v>279.60000000000002</v>
       </c>
-      <c r="C35" s="3">
+      <c r="C35" s="5">
         <v>281.3</v>
       </c>
-      <c r="D35" s="3">
+      <c r="D35" s="5">
         <v>283.5</v>
       </c>
-      <c r="E35" s="3">
+      <c r="E35" s="5">
         <v>285.39999999999998</v>
       </c>
-      <c r="F35" s="3">
+      <c r="F35" s="5">
         <v>285.2</v>
       </c>
-      <c r="G35" s="3">
+      <c r="G35" s="5">
         <v>285.2</v>
       </c>
-      <c r="H35" s="3">
+      <c r="H35" s="5">
         <v>286.5</v>
       </c>
-      <c r="I35" s="3">
+      <c r="I35" s="5">
         <v>288</v>
       </c>
-      <c r="J35" s="3">
+      <c r="J35" s="5">
         <v>291.5</v>
       </c>
-      <c r="K35" s="3">
+      <c r="K35" s="5">
         <v>292.2</v>
       </c>
-      <c r="L35" s="3">
+      <c r="L35" s="5">
         <v>289.8</v>
       </c>
-      <c r="M35" s="3">
+      <c r="M35" s="5">
         <v>288.60000000000002</v>
       </c>
-      <c r="N35" s="3">
+      <c r="N35" s="5">
         <v>286.39999999999998</v>
       </c>
-    </row>
-    <row r="36" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="2">
+      <c r="O35" s="2"/>
+    </row>
+    <row r="36" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="3">
         <v>2006</v>
       </c>
-      <c r="B36" s="3">
+      <c r="B36" s="5">
         <v>290.8</v>
       </c>
-      <c r="C36" s="3">
+      <c r="C36" s="5">
         <v>291.39999999999998</v>
       </c>
-      <c r="D36" s="3">
+      <c r="D36" s="5">
         <v>293.10000000000002</v>
       </c>
-      <c r="E36" s="3">
+      <c r="E36" s="5">
         <v>295.5</v>
       </c>
-      <c r="F36" s="3">
+      <c r="F36" s="5">
         <v>296.89999999999998</v>
       </c>
-      <c r="G36" s="3">
+      <c r="G36" s="5">
         <v>297.60000000000002</v>
       </c>
-      <c r="H36" s="3">
+      <c r="H36" s="5">
         <v>298.39999999999998</v>
       </c>
-      <c r="I36" s="3">
+      <c r="I36" s="5">
         <v>299.10000000000002</v>
       </c>
-      <c r="J36" s="3">
+      <c r="J36" s="5">
         <v>297.60000000000002</v>
       </c>
-      <c r="K36" s="3">
+      <c r="K36" s="5">
         <v>296</v>
       </c>
-      <c r="L36" s="3">
+      <c r="L36" s="5">
         <v>295.60000000000002</v>
       </c>
-      <c r="M36" s="3">
+      <c r="M36" s="5">
         <v>296</v>
       </c>
-      <c r="N36" s="3">
+      <c r="N36" s="5">
         <v>295.7</v>
       </c>
-    </row>
-    <row r="37" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="2">
+      <c r="O36" s="2"/>
+    </row>
+    <row r="37" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="3">
         <v>2007</v>
       </c>
-      <c r="B37" s="3">
+      <c r="B37" s="5">
         <v>296.89999999999998</v>
       </c>
-      <c r="C37" s="3">
+      <c r="C37" s="5">
         <v>298.5</v>
       </c>
-      <c r="D37" s="3">
+      <c r="D37" s="5">
         <v>301.2</v>
       </c>
-      <c r="E37" s="3">
+      <c r="E37" s="5">
         <v>303.10000000000002</v>
       </c>
-      <c r="F37" s="3">
+      <c r="F37" s="5">
         <v>305</v>
       </c>
-      <c r="G37" s="3">
+      <c r="G37" s="5">
         <v>305.60000000000002</v>
       </c>
-      <c r="H37" s="3">
+      <c r="H37" s="5">
         <v>305.5</v>
       </c>
-      <c r="I37" s="3">
+      <c r="I37" s="5">
         <v>304.89999999999998</v>
       </c>
-      <c r="J37" s="3">
+      <c r="J37" s="5">
         <v>305.8</v>
       </c>
-      <c r="K37" s="3">
+      <c r="K37" s="5">
         <v>306.39999999999998</v>
       </c>
-      <c r="L37" s="3">
+      <c r="L37" s="5">
         <v>308.3</v>
       </c>
-      <c r="M37" s="3">
+      <c r="M37" s="5">
         <v>308.10000000000002</v>
       </c>
-      <c r="N37" s="3">
+      <c r="N37" s="5">
         <v>304.10000000000002</v>
       </c>
-    </row>
-    <row r="38" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="2">
+      <c r="O37" s="2"/>
+    </row>
+    <row r="38" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="3">
         <v>2008</v>
       </c>
-      <c r="B38" s="3">
+      <c r="B38" s="5">
         <v>309.60000000000002</v>
       </c>
-      <c r="C38" s="3">
+      <c r="C38" s="5">
         <v>310.5</v>
       </c>
-      <c r="D38" s="3">
+      <c r="D38" s="5">
         <v>313.2</v>
       </c>
-      <c r="E38" s="3">
+      <c r="E38" s="5">
         <v>315.10000000000002</v>
       </c>
-      <c r="F38" s="3">
+      <c r="F38" s="5">
         <v>317.7</v>
       </c>
-      <c r="G38" s="3">
+      <c r="G38" s="5">
         <v>320.89999999999998</v>
       </c>
-      <c r="H38" s="3">
+      <c r="H38" s="5">
         <v>322.60000000000002</v>
       </c>
-      <c r="I38" s="3">
+      <c r="I38" s="5">
         <v>321.3</v>
       </c>
-      <c r="J38" s="3">
+      <c r="J38" s="5">
         <v>320.89999999999998</v>
       </c>
-      <c r="K38" s="3">
+      <c r="K38" s="5">
         <v>317.60000000000002</v>
       </c>
-      <c r="L38" s="3">
+      <c r="L38" s="5">
         <v>311.60000000000002</v>
       </c>
-      <c r="M38" s="3">
+      <c r="M38" s="5">
         <v>308.3</v>
       </c>
-      <c r="N38" s="3">
+      <c r="N38" s="5">
         <v>315.8</v>
       </c>
-    </row>
-    <row r="39" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="2">
+      <c r="O38" s="2"/>
+    </row>
+    <row r="39" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="3">
         <v>2009</v>
       </c>
-      <c r="B39" s="3">
+      <c r="B39" s="5">
         <v>309.7</v>
       </c>
-      <c r="C39" s="3">
+      <c r="C39" s="5">
         <v>311.2</v>
       </c>
-      <c r="D39" s="3">
+      <c r="D39" s="5">
         <v>312</v>
       </c>
-      <c r="E39" s="3">
+      <c r="E39" s="5">
         <v>312.8</v>
       </c>
-      <c r="F39" s="3">
+      <c r="F39" s="5">
         <v>313.7</v>
       </c>
-      <c r="G39" s="3">
+      <c r="G39" s="5">
         <v>316.39999999999998</v>
       </c>
-      <c r="H39" s="3">
+      <c r="H39" s="5">
         <v>315.8</v>
       </c>
-      <c r="I39" s="3">
+      <c r="I39" s="5">
         <v>316.60000000000002</v>
       </c>
-      <c r="J39" s="3">
+      <c r="J39" s="5">
         <v>316.8</v>
       </c>
-      <c r="K39" s="3">
+      <c r="K39" s="5">
         <v>317.10000000000002</v>
       </c>
-      <c r="L39" s="3">
+      <c r="L39" s="5">
         <v>317.3</v>
       </c>
-      <c r="M39" s="3">
+      <c r="M39" s="5">
         <v>316.7</v>
       </c>
-      <c r="N39" s="3">
+      <c r="N39" s="5">
         <v>314.7</v>
       </c>
-    </row>
-    <row r="40" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="2">
+      <c r="O39" s="2"/>
+    </row>
+    <row r="40" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="3">
         <v>2010</v>
       </c>
-      <c r="B40" s="3">
+      <c r="B40" s="5">
         <v>317.8</v>
       </c>
-      <c r="C40" s="3">
+      <c r="C40" s="5">
         <v>317.89999999999998</v>
       </c>
-      <c r="D40" s="3">
+      <c r="D40" s="5">
         <v>319.2</v>
       </c>
-      <c r="E40" s="3">
+      <c r="E40" s="5">
         <v>319.8</v>
       </c>
-      <c r="F40" s="3">
+      <c r="F40" s="5">
         <v>320</v>
       </c>
-      <c r="G40" s="3">
+      <c r="G40" s="5">
         <v>319.7</v>
       </c>
-      <c r="H40" s="3">
+      <c r="H40" s="5">
         <v>319.8</v>
       </c>
-      <c r="I40" s="3">
+      <c r="I40" s="5">
         <v>320.2</v>
       </c>
-      <c r="J40" s="3">
+      <c r="J40" s="5">
         <v>320.39999999999998</v>
       </c>
-      <c r="K40" s="3">
+      <c r="K40" s="5">
         <v>320.8</v>
       </c>
-      <c r="L40" s="3">
+      <c r="L40" s="5">
         <v>320.89999999999998</v>
       </c>
-      <c r="M40" s="3">
+      <c r="M40" s="5">
         <v>321.5</v>
       </c>
-      <c r="N40" s="3">
+      <c r="N40" s="5">
         <v>319.8</v>
       </c>
-    </row>
-    <row r="41" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="2">
+      <c r="O40" s="2"/>
+    </row>
+    <row r="41" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="3">
         <v>2011</v>
       </c>
-      <c r="B41" s="3">
+      <c r="B41" s="5">
         <v>323</v>
       </c>
-      <c r="C41" s="3">
+      <c r="C41" s="5">
         <v>324.60000000000002</v>
       </c>
-      <c r="D41" s="3">
+      <c r="D41" s="5">
         <v>327.8</v>
       </c>
-      <c r="E41" s="3">
+      <c r="E41" s="5">
         <v>329.9</v>
       </c>
-      <c r="F41" s="3">
+      <c r="F41" s="5">
         <v>331.5</v>
       </c>
-      <c r="G41" s="3">
+      <c r="G41" s="5">
         <v>331.1</v>
       </c>
-      <c r="H41" s="3">
+      <c r="H41" s="5">
         <v>331.4</v>
       </c>
-      <c r="I41" s="3">
+      <c r="I41" s="5">
         <v>332.3</v>
       </c>
-      <c r="J41" s="3">
+      <c r="J41" s="5">
         <v>332.8</v>
       </c>
-      <c r="K41" s="3">
+      <c r="K41" s="5">
         <v>332.2</v>
       </c>
-      <c r="L41" s="3">
+      <c r="L41" s="5">
         <v>331.9</v>
       </c>
-      <c r="M41" s="3">
+      <c r="M41" s="5">
         <v>331.1</v>
       </c>
-      <c r="N41" s="3">
+      <c r="N41" s="5">
         <v>330</v>
       </c>
-    </row>
-    <row r="42" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="2">
+      <c r="O41" s="2"/>
+    </row>
+    <row r="42" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="3">
         <v>2012</v>
       </c>
-      <c r="B42" s="3">
+      <c r="B42" s="5">
         <v>332.6</v>
       </c>
-      <c r="C42" s="3">
+      <c r="C42" s="5">
         <v>334</v>
       </c>
-      <c r="D42" s="3">
+      <c r="D42" s="5">
         <v>336.6</v>
       </c>
-      <c r="E42" s="3">
+      <c r="E42" s="5">
         <v>337.6</v>
       </c>
-      <c r="F42" s="3">
+      <c r="F42" s="5">
         <v>337.2</v>
       </c>
-      <c r="G42" s="3">
+      <c r="G42" s="5">
         <v>336.7</v>
       </c>
-      <c r="H42" s="3">
+      <c r="H42" s="5">
         <v>336.2</v>
       </c>
-      <c r="I42" s="3">
+      <c r="I42" s="5">
         <v>338.1</v>
       </c>
-      <c r="J42" s="3">
+      <c r="J42" s="5">
         <v>339.6</v>
       </c>
-      <c r="K42" s="3">
+      <c r="K42" s="5">
         <v>339.5</v>
       </c>
-      <c r="L42" s="3">
+      <c r="L42" s="5">
         <v>337.9</v>
       </c>
-      <c r="M42" s="3">
+      <c r="M42" s="5">
         <v>337</v>
       </c>
-      <c r="N42" s="3">
+      <c r="N42" s="5">
         <v>336.9</v>
       </c>
-    </row>
-    <row r="43" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="2">
+      <c r="O42" s="2"/>
+    </row>
+    <row r="43" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="3">
         <v>2013</v>
       </c>
-      <c r="B43" s="3">
+      <c r="B43" s="5">
         <v>338</v>
       </c>
-      <c r="C43" s="3">
+      <c r="C43" s="5">
         <v>340.8</v>
       </c>
-      <c r="D43" s="3">
+      <c r="D43" s="5">
         <v>341.7</v>
       </c>
-      <c r="E43" s="3">
+      <c r="E43" s="5">
         <v>341.3</v>
       </c>
-      <c r="F43" s="3">
+      <c r="F43" s="5">
         <v>341.9</v>
       </c>
-      <c r="G43" s="3">
+      <c r="G43" s="5">
         <v>342.8</v>
       </c>
-      <c r="H43" s="3">
+      <c r="H43" s="5">
         <v>342.9</v>
       </c>
-      <c r="I43" s="3">
+      <c r="I43" s="5">
         <v>343.3</v>
       </c>
-      <c r="J43" s="3">
+      <c r="J43" s="5">
         <v>343.8</v>
       </c>
-      <c r="K43" s="3">
+      <c r="K43" s="5">
         <v>342.9</v>
       </c>
-      <c r="L43" s="3">
+      <c r="L43" s="5">
         <v>342.2</v>
       </c>
-      <c r="M43" s="3">
+      <c r="M43" s="5">
         <v>342.2</v>
       </c>
-      <c r="N43" s="3">
+      <c r="N43" s="5">
         <v>342</v>
       </c>
-    </row>
-    <row r="44" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="2">
+      <c r="O43" s="2"/>
+    </row>
+    <row r="44" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="3">
         <v>2014</v>
       </c>
-      <c r="B44" s="3">
+      <c r="B44" s="5">
         <v>343.5</v>
       </c>
-      <c r="C44" s="3">
+      <c r="C44" s="5">
         <v>344.8</v>
       </c>
-      <c r="D44" s="3">
+      <c r="D44" s="5">
         <v>347</v>
       </c>
-      <c r="E44" s="3">
+      <c r="E44" s="5">
         <v>348.2</v>
       </c>
-      <c r="F44" s="3">
+      <c r="F44" s="5">
         <v>349.4</v>
       </c>
-      <c r="G44" s="3">
+      <c r="G44" s="5">
         <v>350.1</v>
       </c>
-      <c r="H44" s="3">
+      <c r="H44" s="5">
         <v>349.9</v>
       </c>
-      <c r="I44" s="3">
+      <c r="I44" s="5">
         <v>349.3</v>
       </c>
-      <c r="J44" s="3">
+      <c r="J44" s="5">
         <v>349.6</v>
       </c>
-      <c r="K44" s="3">
+      <c r="K44" s="5">
         <v>348.7</v>
       </c>
-      <c r="L44" s="3">
+      <c r="L44" s="5">
         <v>346.9</v>
       </c>
-      <c r="M44" s="3">
+      <c r="M44" s="5">
         <v>344.9</v>
       </c>
-      <c r="N44" s="3">
+      <c r="N44" s="5">
         <v>347.7</v>
       </c>
-    </row>
-    <row r="45" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="2">
+      <c r="O44" s="2"/>
+    </row>
+    <row r="45" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="3">
         <v>2015</v>
       </c>
-      <c r="B45" s="3">
+      <c r="B45" s="5">
         <v>343.4</v>
       </c>
-      <c r="C45" s="3">
+      <c r="C45" s="5">
         <v>344.9</v>
       </c>
-      <c r="D45" s="3">
+      <c r="D45" s="5">
         <v>346.9</v>
       </c>
-      <c r="E45" s="3">
+      <c r="E45" s="5">
         <v>347.7</v>
       </c>
-      <c r="F45" s="3">
+      <c r="F45" s="5">
         <v>349.4</v>
       </c>
-      <c r="G45" s="3">
+      <c r="G45" s="5">
         <v>350.7</v>
       </c>
-      <c r="H45" s="3">
+      <c r="H45" s="5">
         <v>350.7</v>
       </c>
-      <c r="I45" s="3">
+      <c r="I45" s="5">
         <v>350.2</v>
       </c>
-      <c r="J45" s="3">
+      <c r="J45" s="5">
         <v>349.7</v>
       </c>
-      <c r="K45" s="3">
+      <c r="K45" s="5">
         <v>349.5</v>
       </c>
-      <c r="L45" s="3">
+      <c r="L45" s="5">
         <v>348.8</v>
       </c>
-      <c r="M45" s="3">
+      <c r="M45" s="5">
         <v>347.6</v>
       </c>
-      <c r="N45" s="3">
+      <c r="N45" s="5">
         <v>348.3</v>
       </c>
-    </row>
-    <row r="46" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="2">
+      <c r="O45" s="2"/>
+    </row>
+    <row r="46" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="3">
         <v>2016</v>
       </c>
-      <c r="B46" s="3">
+      <c r="B46" s="5">
         <v>348.2</v>
       </c>
-      <c r="C46" s="3">
+      <c r="C46" s="5">
         <v>348.5</v>
       </c>
-      <c r="D46" s="3">
+      <c r="D46" s="5">
         <v>350</v>
       </c>
-      <c r="E46" s="3">
+      <c r="E46" s="5">
         <v>351.7</v>
       </c>
-      <c r="F46" s="3">
+      <c r="F46" s="5">
         <v>353.1</v>
       </c>
-      <c r="G46" s="3">
+      <c r="G46" s="5">
         <v>354.2</v>
       </c>
-      <c r="H46" s="3">
+      <c r="H46" s="5">
         <v>353.7</v>
       </c>
-      <c r="I46" s="3">
+      <c r="I46" s="5">
         <v>354</v>
       </c>
-      <c r="J46" s="3">
+      <c r="J46" s="5">
         <v>354.8</v>
       </c>
-      <c r="K46" s="3">
+      <c r="K46" s="5">
         <v>355.3</v>
       </c>
-      <c r="L46" s="3">
+      <c r="L46" s="5">
         <v>354.7</v>
       </c>
-      <c r="M46" s="3">
+      <c r="M46" s="5">
         <v>354.9</v>
       </c>
-      <c r="N46" s="3">
+      <c r="N46" s="5">
         <v>352.8</v>
       </c>
-    </row>
-    <row r="47" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="2">
+      <c r="O46" s="2"/>
+    </row>
+    <row r="47" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="3">
         <v>2017</v>
       </c>
-      <c r="B47" s="3">
+      <c r="B47" s="5">
         <v>356.9</v>
       </c>
-      <c r="C47" s="3">
+      <c r="C47" s="5">
         <v>358</v>
       </c>
-      <c r="D47" s="3">
+      <c r="D47" s="5">
         <v>358.3</v>
       </c>
-      <c r="E47" s="3">
+      <c r="E47" s="5">
         <v>359.4</v>
       </c>
-      <c r="F47" s="3">
+      <c r="F47" s="5">
         <v>359.7</v>
       </c>
-      <c r="G47" s="3">
+      <c r="G47" s="5">
         <v>360</v>
       </c>
-      <c r="H47" s="3">
+      <c r="H47" s="5">
         <v>359.8</v>
       </c>
-      <c r="I47" s="3">
+      <c r="I47" s="5">
         <v>360.9</v>
       </c>
-      <c r="J47" s="3">
+      <c r="J47" s="5">
         <v>362.8</v>
       </c>
-      <c r="K47" s="3">
+      <c r="K47" s="5">
         <v>362.5</v>
       </c>
-      <c r="L47" s="3">
+      <c r="L47" s="5">
         <v>362.6</v>
       </c>
-      <c r="M47" s="3">
+      <c r="M47" s="5">
         <v>362.3</v>
       </c>
-      <c r="N47" s="3">
+      <c r="N47" s="5">
         <v>360.3</v>
       </c>
-    </row>
-    <row r="48" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="2">
+      <c r="O47" s="2"/>
+    </row>
+    <row r="48" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="3">
         <v>2018</v>
       </c>
-      <c r="B48" s="3">
+      <c r="B48" s="5">
         <v>364.3</v>
       </c>
-      <c r="C48" s="3">
+      <c r="C48" s="5">
         <v>366</v>
       </c>
-      <c r="D48" s="3">
+      <c r="D48" s="5">
         <v>366.7</v>
       </c>
-      <c r="E48" s="3">
+      <c r="E48" s="5">
         <v>368.3</v>
       </c>
-      <c r="F48" s="3">
+      <c r="F48" s="5">
         <v>369.8</v>
       </c>
-      <c r="G48" s="3">
+      <c r="G48" s="5">
         <v>370.3</v>
       </c>
-      <c r="H48" s="3">
+      <c r="H48" s="5">
         <v>370.4</v>
       </c>
-      <c r="I48" s="3">
+      <c r="I48" s="5">
         <v>370.7</v>
       </c>
-      <c r="J48" s="3">
+      <c r="J48" s="5">
         <v>371.1</v>
       </c>
-      <c r="K48" s="3">
+      <c r="K48" s="5">
         <v>371.8</v>
       </c>
-      <c r="L48" s="3">
+      <c r="L48" s="5">
         <v>370.6</v>
       </c>
-      <c r="M48" s="3">
+      <c r="M48" s="5">
         <v>369.3</v>
       </c>
-      <c r="N48" s="3">
+      <c r="N48" s="5">
         <v>369.1</v>
       </c>
-    </row>
-    <row r="49" spans="1:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="2">
+      <c r="O48" s="2"/>
+    </row>
+    <row r="49" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="3">
         <v>2019</v>
       </c>
-      <c r="B49" s="3">
+      <c r="B49" s="5">
         <v>370</v>
       </c>
-      <c r="C49" s="3">
+      <c r="C49" s="5">
         <v>371.5</v>
       </c>
-      <c r="D49" s="3">
+      <c r="D49" s="5">
         <v>373.6</v>
       </c>
-      <c r="E49" s="3">
+      <c r="E49" s="5">
         <v>375.6</v>
       </c>
-      <c r="F49" s="3">
+      <c r="F49" s="5">
         <v>376.4</v>
       </c>
-      <c r="G49" s="3">
+      <c r="G49" s="5">
         <v>376.5</v>
       </c>
-      <c r="H49" s="3">
+      <c r="H49" s="5">
         <v>377.2</v>
       </c>
-      <c r="I49" s="3">
+      <c r="I49" s="5">
         <v>377.1</v>
       </c>
-      <c r="J49" s="3">
+      <c r="J49" s="5">
         <v>377.5</v>
       </c>
-      <c r="K49" s="3">
+      <c r="K49" s="5">
         <v>378.4</v>
       </c>
-      <c r="L49" s="3">
+      <c r="L49" s="5">
         <v>378.2</v>
       </c>
-      <c r="M49" s="3">
+      <c r="M49" s="5">
         <v>377.8</v>
       </c>
-      <c r="N49" s="3">
+      <c r="N49" s="5">
         <v>375.8</v>
       </c>
-    </row>
-    <row r="50" spans="1:14" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A50" s="2">
+      <c r="O49" s="2"/>
+    </row>
+    <row r="50" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="3">
         <v>2020</v>
       </c>
-      <c r="B50" s="3">
+      <c r="B50" s="5">
         <v>379.2</v>
       </c>
-      <c r="C50" s="3">
+      <c r="C50" s="5">
         <v>380.2</v>
       </c>
-      <c r="D50" s="3">
+      <c r="D50" s="5">
         <v>379.5</v>
       </c>
-      <c r="E50" s="3">
+      <c r="E50" s="5">
         <v>377.2</v>
       </c>
-      <c r="F50" s="3">
+      <c r="F50" s="5">
         <v>377.2</v>
       </c>
-      <c r="G50" s="3">
+      <c r="G50" s="5">
         <v>379.4</v>
       </c>
-      <c r="H50" s="3">
+      <c r="H50" s="5">
         <v>381.3</v>
       </c>
-      <c r="I50" s="3">
+      <c r="I50" s="5">
         <v>382.6</v>
       </c>
-      <c r="J50" s="3">
+      <c r="J50" s="5">
         <v>383.1</v>
       </c>
-      <c r="K50" s="3">
+      <c r="K50" s="5">
         <v>383.2</v>
       </c>
-      <c r="L50" s="3">
+      <c r="L50" s="5">
         <v>382.9</v>
       </c>
-      <c r="M50" s="3">
+      <c r="M50" s="5">
         <v>383.2</v>
       </c>
-      <c r="N50" s="3">
+      <c r="N50" s="5">
         <v>380.8</v>
       </c>
-    </row>
-    <row r="51" spans="1:14" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A51" s="2">
+      <c r="O50" s="2"/>
+    </row>
+    <row r="51" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="3">
         <v>2021</v>
       </c>
-      <c r="B51" s="3">
+      <c r="B51" s="5">
         <v>384.9</v>
       </c>
-      <c r="C51" s="3">
+      <c r="C51" s="5">
         <v>387.1</v>
       </c>
-      <c r="D51" s="3">
+      <c r="D51" s="5">
         <v>390</v>
       </c>
-      <c r="E51" s="3">
+      <c r="E51" s="5">
         <v>393.2</v>
       </c>
-      <c r="F51" s="3">
+      <c r="F51" s="5">
         <v>396.7</v>
       </c>
-      <c r="G51" s="3">
+      <c r="G51" s="5">
         <v>400.5</v>
       </c>
-      <c r="H51" s="3">
+      <c r="H51" s="5">
         <v>402.4</v>
       </c>
-      <c r="I51" s="3">
+      <c r="I51" s="5">
         <v>403.1</v>
       </c>
-      <c r="J51" s="3">
+      <c r="J51" s="5">
         <v>404.2</v>
       </c>
-      <c r="K51" s="3">
+      <c r="K51" s="5">
         <v>407.6</v>
       </c>
-      <c r="L51" s="3">
+      <c r="L51" s="5">
         <v>409.5</v>
       </c>
-      <c r="M51" s="3">
+      <c r="M51" s="5">
         <v>410.8</v>
       </c>
-      <c r="N51" s="3">
+      <c r="N51" s="5">
         <v>399.2</v>
       </c>
-    </row>
-    <row r="52" spans="1:14" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A52" s="6">
+      <c r="O51" s="2"/>
+    </row>
+    <row r="52" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="3">
         <v>2022</v>
       </c>
-      <c r="B52" s="7">
+      <c r="B52" s="5">
         <v>414.3</v>
       </c>
-      <c r="C52" s="7">
+      <c r="C52" s="5">
         <v>418.2</v>
       </c>
-      <c r="D52" s="7">
+      <c r="D52" s="5">
         <v>423.9</v>
       </c>
-      <c r="E52" s="7">
+      <c r="E52" s="5">
         <v>426.3</v>
       </c>
-      <c r="F52" s="7">
+      <c r="F52" s="5">
         <v>431</v>
       </c>
-      <c r="G52" s="7">
+      <c r="G52" s="5">
         <v>436.9</v>
       </c>
-      <c r="H52" s="7">
+      <c r="H52" s="5">
         <v>436.8</v>
       </c>
-      <c r="I52" s="7">
+      <c r="I52" s="5">
         <v>436.7</v>
       </c>
-      <c r="J52" s="7">
+      <c r="J52" s="5">
         <v>437.6</v>
       </c>
-      <c r="K52" s="7">
+      <c r="K52" s="5">
         <v>439.4</v>
       </c>
-      <c r="L52" s="7">
+      <c r="L52" s="5">
         <v>439</v>
       </c>
-      <c r="M52" s="7">
+      <c r="M52" s="5">
         <v>437.6</v>
       </c>
-      <c r="N52" s="7">
+      <c r="N52" s="5">
         <v>431.5</v>
       </c>
-    </row>
-    <row r="53" spans="1:14" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A53" s="1">
+      <c r="O52" s="2"/>
+    </row>
+    <row r="53" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="3">
         <v>2023</v>
       </c>
-      <c r="B53" s="7">
+      <c r="B53" s="5">
         <v>441.1</v>
       </c>
-      <c r="C53" s="7">
+      <c r="C53" s="5">
         <v>443.6</v>
       </c>
-      <c r="D53" s="7">
+      <c r="D53" s="5">
         <v>445</v>
       </c>
-      <c r="E53" s="7">
+      <c r="E53" s="5">
         <v>447.3</v>
       </c>
-      <c r="F53" s="7">
+      <c r="F53" s="5">
         <v>448.4</v>
       </c>
-      <c r="G53" s="7">
+      <c r="G53" s="5">
         <v>449.9</v>
       </c>
-      <c r="H53" s="7">
+      <c r="H53" s="5">
         <v>450.7</v>
       </c>
-      <c r="I53" s="7">
+      <c r="I53" s="5">
         <v>452.7</v>
       </c>
-      <c r="J53" s="7">
+      <c r="J53" s="5">
         <v>453.8</v>
       </c>
-      <c r="K53" s="7">
+      <c r="K53" s="5">
         <v>453.6</v>
       </c>
-      <c r="L53" s="7">
+      <c r="L53" s="5">
         <v>452.7</v>
       </c>
-      <c r="M53" s="7">
+      <c r="M53" s="5">
         <v>452.3</v>
       </c>
-      <c r="N53" s="7">
+      <c r="N53" s="5">
         <v>449.3</v>
       </c>
+      <c r="O53" s="2"/>
+    </row>
+    <row r="54" spans="1:15" ht="12.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="3">
+        <v>2024</v>
+      </c>
+      <c r="B54" s="5">
+        <v>454.7</v>
+      </c>
+      <c r="C54" s="5">
+        <v>457.6</v>
+      </c>
+      <c r="D54" s="5">
+        <v>460.5</v>
+      </c>
+      <c r="E54" s="5">
+        <v>462.3</v>
+      </c>
+      <c r="F54" s="5">
+        <v>463.1</v>
+      </c>
+      <c r="G54" s="5">
+        <v>463.2</v>
+      </c>
+      <c r="H54" s="5">
+        <v>463.8</v>
+      </c>
+      <c r="I54" s="5">
+        <v>464.1</v>
+      </c>
+      <c r="J54" s="5">
+        <v>464.9</v>
+      </c>
+      <c r="K54" s="5">
+        <v>465.4</v>
+      </c>
+      <c r="L54" s="5">
+        <v>465.2</v>
+      </c>
+      <c r="M54" s="5">
+        <v>465.3</v>
+      </c>
+      <c r="N54" s="5">
+        <v>462.5</v>
+      </c>
+      <c r="O54" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update cpi_u_rs with 2025 data
</commit_message>
<xml_diff>
--- a/data-raw/cpi_u_rs.xlsx
+++ b/data-raw/cpi_u_rs.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\March 2025\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Website\Website Updates\2026\R-CPI-U-RS\run 2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCD3BFA0-4106-4EDE-85AC-1E3C92BA40FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{642F9DC8-29D5-47CB-B132-E626BD0D4595}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-135" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="All items" sheetId="1" r:id="rId1"/>
+    <sheet name="All items" sheetId="2" r:id="rId1"/>
   </sheets>
   <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>YEAR</t>
   </si>
@@ -78,6 +78,12 @@
   <si>
     <t>December 1977=100</t>
   </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Note: The Oct 2025 data values are not available due to the 2025 lapse in appropriations.</t>
+  </si>
 </sst>
 </file>
 
@@ -94,7 +100,7 @@
       <charset val="204"/>
     </font>
     <font>
-      <sz val="11"/>
+      <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -102,14 +108,16 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
+      <sz val="10"/>
+      <color rgb="FF333333"/>
+      <name val="Tahoma"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -133,39 +141,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -473,2267 +463,2208 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O54"/>
-  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09018F99-0D91-49BB-84FC-143CA7E814CE}">
+  <dimension ref="A1:N57"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="6.88671875" customWidth="1"/>
-    <col min="2" max="6" width="5.77734375" customWidth="1"/>
-    <col min="7" max="7" width="6.88671875" customWidth="1"/>
-    <col min="8" max="8" width="5.77734375" customWidth="1"/>
-    <col min="9" max="9" width="6.88671875" customWidth="1"/>
-    <col min="10" max="13" width="5.77734375" customWidth="1"/>
-    <col min="14" max="14" width="5.5546875" customWidth="1"/>
-    <col min="15" max="15" width="51.33203125" customWidth="1"/>
+    <col min="1" max="1" width="9.33203125" style="1"/>
+    <col min="2" max="14" width="9.33203125" style="3"/>
+    <col min="15" max="16384" width="9.33203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
-      <c r="I1" s="10"/>
-      <c r="J1" s="10"/>
-      <c r="K1" s="10"/>
-      <c r="L1" s="10"/>
-      <c r="M1" s="10"/>
-      <c r="N1" s="10"/>
-      <c r="O1" s="10"/>
-    </row>
-    <row r="2" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="10" t="s">
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
-      <c r="I2" s="10"/>
-      <c r="J2" s="10"/>
-      <c r="K2" s="10"/>
-      <c r="L2" s="10"/>
-      <c r="M2" s="10"/>
-      <c r="N2" s="10"/>
-      <c r="O2" s="10"/>
-    </row>
-    <row r="3" spans="1:15" s="10" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="10" t="s">
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="11" t="s">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="10"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10"/>
-      <c r="H4" s="10"/>
-      <c r="I4" s="10"/>
-      <c r="J4" s="10"/>
-      <c r="K4" s="10"/>
-      <c r="L4" s="10"/>
-      <c r="M4" s="10"/>
-      <c r="N4" s="10"/>
-      <c r="O4" s="10"/>
-    </row>
-    <row r="5" spans="1:15" s="10" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="10" t="s">
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:15" s="9" customFormat="1" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="6" t="s">
+    <row r="6" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F6" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="G6" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="H6" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="I6" s="7" t="s">
+      <c r="I6" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="J6" s="7" t="s">
+      <c r="J6" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K6" s="7" t="s">
+      <c r="K6" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="L6" s="7" t="s">
+      <c r="L6" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="M6" s="7" t="s">
+      <c r="M6" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="N6" s="7" t="s">
+      <c r="N6" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="O6" s="8"/>
-    </row>
-    <row r="7" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="3">
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A7" s="1">
         <v>1977</v>
       </c>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
-      <c r="I7" s="4"/>
-      <c r="J7" s="4"/>
-      <c r="K7" s="4"/>
-      <c r="L7" s="4"/>
-      <c r="M7" s="5">
+      <c r="M7" s="3">
         <v>100</v>
       </c>
-      <c r="N7" s="4"/>
-      <c r="O7" s="2"/>
-    </row>
-    <row r="8" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="3">
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A8" s="1">
         <v>1978</v>
       </c>
-      <c r="B8" s="5">
+      <c r="B8" s="3">
         <v>100.5</v>
       </c>
-      <c r="C8" s="5">
+      <c r="C8" s="3">
         <v>101.1</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D8" s="3">
         <v>101.8</v>
       </c>
-      <c r="E8" s="5">
+      <c r="E8" s="3">
         <v>102.7</v>
       </c>
-      <c r="F8" s="5">
+      <c r="F8" s="3">
         <v>103.6</v>
       </c>
-      <c r="G8" s="5">
+      <c r="G8" s="3">
         <v>104.5</v>
       </c>
-      <c r="H8" s="5">
+      <c r="H8" s="3">
         <v>105</v>
       </c>
-      <c r="I8" s="5">
+      <c r="I8" s="3">
         <v>105.5</v>
       </c>
-      <c r="J8" s="5">
+      <c r="J8" s="3">
         <v>106.1</v>
       </c>
-      <c r="K8" s="5">
+      <c r="K8" s="3">
         <v>106.7</v>
       </c>
-      <c r="L8" s="5">
+      <c r="L8" s="3">
         <v>107.3</v>
       </c>
-      <c r="M8" s="5">
+      <c r="M8" s="3">
         <v>107.8</v>
       </c>
-      <c r="N8" s="5">
+      <c r="N8" s="3">
         <v>104.4</v>
       </c>
-      <c r="O8" s="2"/>
-    </row>
-    <row r="9" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="3">
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A9" s="1">
         <v>1979</v>
       </c>
-      <c r="B9" s="5">
+      <c r="B9" s="3">
         <v>108.7</v>
       </c>
-      <c r="C9" s="5">
+      <c r="C9" s="3">
         <v>109.7</v>
       </c>
-      <c r="D9" s="5">
+      <c r="D9" s="3">
         <v>110.7</v>
       </c>
-      <c r="E9" s="5">
+      <c r="E9" s="3">
         <v>111.8</v>
       </c>
-      <c r="F9" s="5">
+      <c r="F9" s="3">
         <v>113</v>
       </c>
-      <c r="G9" s="5">
+      <c r="G9" s="3">
         <v>114.1</v>
       </c>
-      <c r="H9" s="5">
+      <c r="H9" s="3">
         <v>115.1</v>
       </c>
-      <c r="I9" s="5">
+      <c r="I9" s="3">
         <v>116</v>
       </c>
-      <c r="J9" s="5">
+      <c r="J9" s="3">
         <v>117.1</v>
       </c>
-      <c r="K9" s="5">
+      <c r="K9" s="3">
         <v>117.9</v>
       </c>
-      <c r="L9" s="5">
+      <c r="L9" s="3">
         <v>118.5</v>
       </c>
-      <c r="M9" s="5">
+      <c r="M9" s="3">
         <v>119.5</v>
       </c>
-      <c r="N9" s="5">
+      <c r="N9" s="3">
         <v>114.3</v>
       </c>
-      <c r="O9" s="2"/>
-    </row>
-    <row r="10" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="3">
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A10" s="1">
         <v>1980</v>
       </c>
-      <c r="B10" s="5">
+      <c r="B10" s="3">
         <v>120.8</v>
       </c>
-      <c r="C10" s="5">
+      <c r="C10" s="3">
         <v>122.4</v>
       </c>
-      <c r="D10" s="5">
+      <c r="D10" s="3">
         <v>123.8</v>
       </c>
-      <c r="E10" s="5">
+      <c r="E10" s="3">
         <v>124.7</v>
       </c>
-      <c r="F10" s="5">
+      <c r="F10" s="3">
         <v>125.7</v>
       </c>
-      <c r="G10" s="5">
+      <c r="G10" s="3">
         <v>126.7</v>
       </c>
-      <c r="H10" s="5">
+      <c r="H10" s="3">
         <v>127.5</v>
       </c>
-      <c r="I10" s="5">
+      <c r="I10" s="3">
         <v>128.6</v>
       </c>
-      <c r="J10" s="5">
+      <c r="J10" s="3">
         <v>129.9</v>
       </c>
-      <c r="K10" s="5">
+      <c r="K10" s="3">
         <v>130.69999999999999</v>
       </c>
-      <c r="L10" s="5">
+      <c r="L10" s="3">
         <v>131.5</v>
       </c>
-      <c r="M10" s="5">
+      <c r="M10" s="3">
         <v>132.4</v>
       </c>
-      <c r="N10" s="5">
+      <c r="N10" s="3">
         <v>127.1</v>
       </c>
-      <c r="O10" s="2"/>
-    </row>
-    <row r="11" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="3">
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A11" s="1">
         <v>1981</v>
       </c>
-      <c r="B11" s="5">
+      <c r="B11" s="3">
         <v>133.6</v>
       </c>
-      <c r="C11" s="5">
+      <c r="C11" s="3">
         <v>135.19999999999999</v>
       </c>
-      <c r="D11" s="5">
+      <c r="D11" s="3">
         <v>136.30000000000001</v>
       </c>
-      <c r="E11" s="5">
+      <c r="E11" s="3">
         <v>137.1</v>
       </c>
-      <c r="F11" s="5">
+      <c r="F11" s="3">
         <v>137.9</v>
       </c>
-      <c r="G11" s="5">
+      <c r="G11" s="3">
         <v>138.69999999999999</v>
       </c>
-      <c r="H11" s="5">
+      <c r="H11" s="3">
         <v>139.69999999999999</v>
       </c>
-      <c r="I11" s="5">
+      <c r="I11" s="3">
         <v>140.69999999999999</v>
       </c>
-      <c r="J11" s="5">
+      <c r="J11" s="3">
         <v>141.80000000000001</v>
       </c>
-      <c r="K11" s="5">
+      <c r="K11" s="3">
         <v>142.4</v>
       </c>
-      <c r="L11" s="5">
+      <c r="L11" s="3">
         <v>142.9</v>
       </c>
-      <c r="M11" s="5">
+      <c r="M11" s="3">
         <v>143.4</v>
       </c>
-      <c r="N11" s="5">
+      <c r="N11" s="3">
         <v>139.1</v>
       </c>
-      <c r="O11" s="2"/>
-    </row>
-    <row r="12" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="3">
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A12" s="1">
         <v>1982</v>
       </c>
-      <c r="B12" s="5">
+      <c r="B12" s="3">
         <v>144.19999999999999</v>
       </c>
-      <c r="C12" s="5">
+      <c r="C12" s="3">
         <v>144.69999999999999</v>
       </c>
-      <c r="D12" s="5">
+      <c r="D12" s="3">
         <v>144.9</v>
       </c>
-      <c r="E12" s="5">
+      <c r="E12" s="3">
         <v>145</v>
       </c>
-      <c r="F12" s="5">
+      <c r="F12" s="3">
         <v>146.1</v>
       </c>
-      <c r="G12" s="5">
+      <c r="G12" s="3">
         <v>147.5</v>
       </c>
-      <c r="H12" s="5">
+      <c r="H12" s="3">
         <v>148.5</v>
       </c>
-      <c r="I12" s="5">
+      <c r="I12" s="3">
         <v>148.80000000000001</v>
       </c>
-      <c r="J12" s="5">
+      <c r="J12" s="3">
         <v>149.5</v>
       </c>
-      <c r="K12" s="5">
+      <c r="K12" s="3">
         <v>150.19999999999999</v>
       </c>
-      <c r="L12" s="5">
+      <c r="L12" s="3">
         <v>150.5</v>
       </c>
-      <c r="M12" s="5">
+      <c r="M12" s="3">
         <v>150.6</v>
       </c>
-      <c r="N12" s="5">
+      <c r="N12" s="3">
         <v>147.5</v>
       </c>
-      <c r="O12" s="2"/>
-    </row>
-    <row r="13" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="3">
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A13" s="1">
         <v>1983</v>
       </c>
-      <c r="B13" s="5">
+      <c r="B13" s="3">
         <v>151</v>
       </c>
-      <c r="C13" s="5">
+      <c r="C13" s="3">
         <v>151.1</v>
       </c>
-      <c r="D13" s="5">
+      <c r="D13" s="3">
         <v>151.19999999999999</v>
       </c>
-      <c r="E13" s="5">
+      <c r="E13" s="3">
         <v>152.4</v>
       </c>
-      <c r="F13" s="5">
+      <c r="F13" s="3">
         <v>153.19999999999999</v>
       </c>
-      <c r="G13" s="5">
+      <c r="G13" s="3">
         <v>153.69999999999999</v>
       </c>
-      <c r="H13" s="5">
+      <c r="H13" s="3">
         <v>154.30000000000001</v>
       </c>
-      <c r="I13" s="5">
+      <c r="I13" s="3">
         <v>154.80000000000001</v>
       </c>
-      <c r="J13" s="5">
+      <c r="J13" s="3">
         <v>155.6</v>
       </c>
-      <c r="K13" s="5">
+      <c r="K13" s="3">
         <v>156</v>
       </c>
-      <c r="L13" s="5">
+      <c r="L13" s="3">
         <v>156.1</v>
       </c>
-      <c r="M13" s="5">
+      <c r="M13" s="3">
         <v>156.30000000000001</v>
       </c>
-      <c r="N13" s="5">
+      <c r="N13" s="3">
         <v>153.80000000000001</v>
       </c>
-      <c r="O13" s="2"/>
-    </row>
-    <row r="14" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="3">
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A14" s="1">
         <v>1984</v>
       </c>
-      <c r="B14" s="5">
+      <c r="B14" s="3">
         <v>157.19999999999999</v>
       </c>
-      <c r="C14" s="5">
+      <c r="C14" s="3">
         <v>158</v>
       </c>
-      <c r="D14" s="5">
+      <c r="D14" s="3">
         <v>158.30000000000001</v>
       </c>
-      <c r="E14" s="5">
+      <c r="E14" s="3">
         <v>159</v>
       </c>
-      <c r="F14" s="5">
+      <c r="F14" s="3">
         <v>159.5</v>
       </c>
-      <c r="G14" s="5">
+      <c r="G14" s="3">
         <v>159.9</v>
       </c>
-      <c r="H14" s="5">
+      <c r="H14" s="3">
         <v>160.4</v>
       </c>
-      <c r="I14" s="5">
+      <c r="I14" s="3">
         <v>161.1</v>
       </c>
-      <c r="J14" s="5">
+      <c r="J14" s="3">
         <v>161.80000000000001</v>
       </c>
-      <c r="K14" s="5">
+      <c r="K14" s="3">
         <v>162.19999999999999</v>
       </c>
-      <c r="L14" s="5">
+      <c r="L14" s="3">
         <v>162.19999999999999</v>
       </c>
-      <c r="M14" s="5">
+      <c r="M14" s="3">
         <v>162.30000000000001</v>
       </c>
-      <c r="N14" s="5">
+      <c r="N14" s="3">
         <v>160.19999999999999</v>
       </c>
-      <c r="O14" s="2"/>
-    </row>
-    <row r="15" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="3">
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A15" s="1">
         <v>1985</v>
       </c>
-      <c r="B15" s="5">
+      <c r="B15" s="3">
         <v>162.5</v>
       </c>
-      <c r="C15" s="5">
+      <c r="C15" s="3">
         <v>163.19999999999999</v>
       </c>
-      <c r="D15" s="5">
+      <c r="D15" s="3">
         <v>163.9</v>
       </c>
-      <c r="E15" s="5">
+      <c r="E15" s="3">
         <v>164.6</v>
       </c>
-      <c r="F15" s="5">
+      <c r="F15" s="3">
         <v>165.2</v>
       </c>
-      <c r="G15" s="5">
+      <c r="G15" s="3">
         <v>165.6</v>
       </c>
-      <c r="H15" s="5">
+      <c r="H15" s="3">
         <v>165.9</v>
       </c>
-      <c r="I15" s="5">
+      <c r="I15" s="3">
         <v>166.2</v>
       </c>
-      <c r="J15" s="5">
+      <c r="J15" s="3">
         <v>166.8</v>
       </c>
-      <c r="K15" s="5">
+      <c r="K15" s="3">
         <v>167.2</v>
       </c>
-      <c r="L15" s="5">
+      <c r="L15" s="3">
         <v>167.7</v>
       </c>
-      <c r="M15" s="5">
+      <c r="M15" s="3">
         <v>168.1</v>
       </c>
-      <c r="N15" s="5">
+      <c r="N15" s="3">
         <v>165.6</v>
       </c>
-      <c r="O15" s="2"/>
-    </row>
-    <row r="16" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="3">
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A16" s="1">
         <v>1986</v>
       </c>
-      <c r="B16" s="5">
+      <c r="B16" s="3">
         <v>168.6</v>
       </c>
-      <c r="C16" s="5">
+      <c r="C16" s="3">
         <v>168.1</v>
       </c>
-      <c r="D16" s="5">
+      <c r="D16" s="3">
         <v>167.3</v>
       </c>
-      <c r="E16" s="5">
+      <c r="E16" s="3">
         <v>166.9</v>
       </c>
-      <c r="F16" s="5">
+      <c r="F16" s="3">
         <v>167.4</v>
       </c>
-      <c r="G16" s="5">
+      <c r="G16" s="3">
         <v>168.2</v>
       </c>
-      <c r="H16" s="5">
+      <c r="H16" s="3">
         <v>168.2</v>
       </c>
-      <c r="I16" s="5">
+      <c r="I16" s="3">
         <v>168.5</v>
       </c>
-      <c r="J16" s="5">
+      <c r="J16" s="3">
         <v>169.4</v>
       </c>
-      <c r="K16" s="5">
+      <c r="K16" s="3">
         <v>169.5</v>
       </c>
-      <c r="L16" s="5">
+      <c r="L16" s="3">
         <v>169.5</v>
       </c>
-      <c r="M16" s="5">
+      <c r="M16" s="3">
         <v>169.6</v>
       </c>
-      <c r="N16" s="5">
+      <c r="N16" s="3">
         <v>168.4</v>
       </c>
-      <c r="O16" s="2"/>
-    </row>
-    <row r="17" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="3">
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A17" s="1">
         <v>1987</v>
       </c>
-      <c r="B17" s="5">
+      <c r="B17" s="3">
         <v>170.6</v>
       </c>
-      <c r="C17" s="5">
+      <c r="C17" s="3">
         <v>171.3</v>
       </c>
-      <c r="D17" s="5">
+      <c r="D17" s="3">
         <v>172</v>
       </c>
-      <c r="E17" s="5">
+      <c r="E17" s="3">
         <v>172.9</v>
       </c>
-      <c r="F17" s="5">
+      <c r="F17" s="3">
         <v>173.4</v>
       </c>
-      <c r="G17" s="5">
+      <c r="G17" s="3">
         <v>174</v>
       </c>
-      <c r="H17" s="5">
+      <c r="H17" s="3">
         <v>174.3</v>
       </c>
-      <c r="I17" s="5">
+      <c r="I17" s="3">
         <v>175.3</v>
       </c>
-      <c r="J17" s="5">
+      <c r="J17" s="3">
         <v>176.1</v>
       </c>
-      <c r="K17" s="5">
+      <c r="K17" s="3">
         <v>176.5</v>
       </c>
-      <c r="L17" s="5">
+      <c r="L17" s="3">
         <v>176.6</v>
       </c>
-      <c r="M17" s="5">
+      <c r="M17" s="3">
         <v>176.5</v>
       </c>
-      <c r="N17" s="5">
+      <c r="N17" s="3">
         <v>174.1</v>
       </c>
-      <c r="O17" s="2"/>
-    </row>
-    <row r="18" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="3">
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A18" s="1">
         <v>1988</v>
       </c>
-      <c r="B18" s="5">
+      <c r="B18" s="3">
         <v>177</v>
       </c>
-      <c r="C18" s="5">
+      <c r="C18" s="3">
         <v>177.3</v>
       </c>
-      <c r="D18" s="5">
+      <c r="D18" s="3">
         <v>178</v>
       </c>
-      <c r="E18" s="5">
+      <c r="E18" s="3">
         <v>178.9</v>
       </c>
-      <c r="F18" s="5">
+      <c r="F18" s="3">
         <v>179.5</v>
       </c>
-      <c r="G18" s="5">
+      <c r="G18" s="3">
         <v>180.1</v>
       </c>
-      <c r="H18" s="5">
+      <c r="H18" s="3">
         <v>180.8</v>
       </c>
-      <c r="I18" s="5">
+      <c r="I18" s="3">
         <v>181.6</v>
       </c>
-      <c r="J18" s="5">
+      <c r="J18" s="3">
         <v>182.7</v>
       </c>
-      <c r="K18" s="5">
+      <c r="K18" s="3">
         <v>183.2</v>
       </c>
-      <c r="L18" s="5">
+      <c r="L18" s="3">
         <v>183.3</v>
       </c>
-      <c r="M18" s="5">
+      <c r="M18" s="3">
         <v>183.4</v>
       </c>
-      <c r="N18" s="5">
+      <c r="N18" s="3">
         <v>180.5</v>
       </c>
-      <c r="O18" s="2"/>
-    </row>
-    <row r="19" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="3">
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A19" s="1">
         <v>1989</v>
       </c>
-      <c r="B19" s="5">
+      <c r="B19" s="3">
         <v>184.3</v>
       </c>
-      <c r="C19" s="5">
+      <c r="C19" s="3">
         <v>184.9</v>
       </c>
-      <c r="D19" s="5">
+      <c r="D19" s="3">
         <v>185.9</v>
       </c>
-      <c r="E19" s="5">
+      <c r="E19" s="3">
         <v>187.2</v>
       </c>
-      <c r="F19" s="5">
+      <c r="F19" s="3">
         <v>188.1</v>
       </c>
-      <c r="G19" s="5">
+      <c r="G19" s="3">
         <v>188.5</v>
       </c>
-      <c r="H19" s="5">
+      <c r="H19" s="3">
         <v>189</v>
       </c>
-      <c r="I19" s="5">
+      <c r="I19" s="3">
         <v>189.2</v>
       </c>
-      <c r="J19" s="5">
+      <c r="J19" s="3">
         <v>189.8</v>
       </c>
-      <c r="K19" s="5">
+      <c r="K19" s="3">
         <v>190.6</v>
       </c>
-      <c r="L19" s="5">
+      <c r="L19" s="3">
         <v>190.9</v>
       </c>
-      <c r="M19" s="5">
+      <c r="M19" s="3">
         <v>191.1</v>
       </c>
-      <c r="N19" s="5">
+      <c r="N19" s="3">
         <v>188.3</v>
       </c>
-      <c r="O19" s="2"/>
-    </row>
-    <row r="20" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="3">
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A20" s="1">
         <v>1990</v>
       </c>
-      <c r="B20" s="5">
+      <c r="B20" s="3">
         <v>193</v>
       </c>
-      <c r="C20" s="5">
+      <c r="C20" s="3">
         <v>193.9</v>
       </c>
-      <c r="D20" s="5">
+      <c r="D20" s="3">
         <v>194.9</v>
       </c>
-      <c r="E20" s="5">
+      <c r="E20" s="3">
         <v>195.2</v>
       </c>
-      <c r="F20" s="5">
+      <c r="F20" s="3">
         <v>195.5</v>
       </c>
-      <c r="G20" s="5">
+      <c r="G20" s="3">
         <v>196.5</v>
       </c>
-      <c r="H20" s="5">
+      <c r="H20" s="3">
         <v>197.3</v>
       </c>
-      <c r="I20" s="5">
+      <c r="I20" s="3">
         <v>199</v>
       </c>
-      <c r="J20" s="5">
+      <c r="J20" s="3">
         <v>200.6</v>
       </c>
-      <c r="K20" s="5">
+      <c r="K20" s="3">
         <v>201.7</v>
       </c>
-      <c r="L20" s="5">
+      <c r="L20" s="3">
         <v>202</v>
       </c>
-      <c r="M20" s="5">
+      <c r="M20" s="3">
         <v>202</v>
       </c>
-      <c r="N20" s="5">
+      <c r="N20" s="3">
         <v>197.6</v>
       </c>
-      <c r="O20" s="2"/>
-    </row>
-    <row r="21" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="3">
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A21" s="1">
         <v>1991</v>
       </c>
-      <c r="B21" s="5">
+      <c r="B21" s="3">
         <v>202.9</v>
       </c>
-      <c r="C21" s="5">
+      <c r="C21" s="3">
         <v>203.1</v>
       </c>
-      <c r="D21" s="5">
+      <c r="D21" s="3">
         <v>203.3</v>
       </c>
-      <c r="E21" s="5">
+      <c r="E21" s="3">
         <v>203.5</v>
       </c>
-      <c r="F21" s="5">
+      <c r="F21" s="3">
         <v>204.1</v>
       </c>
-      <c r="G21" s="5">
+      <c r="G21" s="3">
         <v>204.5</v>
       </c>
-      <c r="H21" s="5">
+      <c r="H21" s="3">
         <v>204.7</v>
       </c>
-      <c r="I21" s="5">
+      <c r="I21" s="3">
         <v>205.2</v>
       </c>
-      <c r="J21" s="5">
+      <c r="J21" s="3">
         <v>206.1</v>
       </c>
-      <c r="K21" s="5">
+      <c r="K21" s="3">
         <v>206.2</v>
       </c>
-      <c r="L21" s="5">
+      <c r="L21" s="3">
         <v>206.7</v>
       </c>
-      <c r="M21" s="5">
+      <c r="M21" s="3">
         <v>206.8</v>
       </c>
-      <c r="N21" s="5">
+      <c r="N21" s="3">
         <v>204.8</v>
       </c>
-      <c r="O21" s="2"/>
-    </row>
-    <row r="22" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="3">
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A22" s="1">
         <v>1992</v>
       </c>
-      <c r="B22" s="5">
+      <c r="B22" s="3">
         <v>207.2</v>
       </c>
-      <c r="C22" s="5">
+      <c r="C22" s="3">
         <v>207.7</v>
       </c>
-      <c r="D22" s="5">
+      <c r="D22" s="3">
         <v>208.6</v>
       </c>
-      <c r="E22" s="5">
+      <c r="E22" s="3">
         <v>209</v>
       </c>
-      <c r="F22" s="5">
+      <c r="F22" s="3">
         <v>209.3</v>
       </c>
-      <c r="G22" s="5">
+      <c r="G22" s="3">
         <v>209.7</v>
       </c>
-      <c r="H22" s="5">
+      <c r="H22" s="3">
         <v>210.1</v>
       </c>
-      <c r="I22" s="5">
+      <c r="I22" s="3">
         <v>210.6</v>
       </c>
-      <c r="J22" s="5">
+      <c r="J22" s="3">
         <v>211.2</v>
       </c>
-      <c r="K22" s="5">
+      <c r="K22" s="3">
         <v>211.8</v>
       </c>
-      <c r="L22" s="5">
+      <c r="L22" s="3">
         <v>212.1</v>
       </c>
-      <c r="M22" s="5">
+      <c r="M22" s="3">
         <v>211.9</v>
       </c>
-      <c r="N22" s="5">
+      <c r="N22" s="3">
         <v>209.9</v>
       </c>
-      <c r="O22" s="2"/>
-    </row>
-    <row r="23" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="3">
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A23" s="1">
         <v>1993</v>
       </c>
-      <c r="B23" s="5">
+      <c r="B23" s="3">
         <v>212.6</v>
       </c>
-      <c r="C23" s="5">
+      <c r="C23" s="3">
         <v>213.3</v>
       </c>
-      <c r="D23" s="5">
+      <c r="D23" s="3">
         <v>214</v>
       </c>
-      <c r="E23" s="5">
+      <c r="E23" s="3">
         <v>214.5</v>
       </c>
-      <c r="F23" s="5">
+      <c r="F23" s="3">
         <v>215</v>
       </c>
-      <c r="G23" s="5">
+      <c r="G23" s="3">
         <v>215.2</v>
       </c>
-      <c r="H23" s="5">
+      <c r="H23" s="3">
         <v>215.3</v>
       </c>
-      <c r="I23" s="5">
+      <c r="I23" s="3">
         <v>215.7</v>
       </c>
-      <c r="J23" s="5">
+      <c r="J23" s="3">
         <v>216</v>
       </c>
-      <c r="K23" s="5">
+      <c r="K23" s="3">
         <v>216.7</v>
       </c>
-      <c r="L23" s="5">
+      <c r="L23" s="3">
         <v>216.9</v>
       </c>
-      <c r="M23" s="5">
+      <c r="M23" s="3">
         <v>216.7</v>
       </c>
-      <c r="N23" s="5">
+      <c r="N23" s="3">
         <v>215.2</v>
       </c>
-      <c r="O23" s="2"/>
-    </row>
-    <row r="24" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="3">
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A24" s="1">
         <v>1994</v>
       </c>
-      <c r="B24" s="5">
+      <c r="B24" s="3">
         <v>217.1</v>
       </c>
-      <c r="C24" s="5">
+      <c r="C24" s="3">
         <v>217.6</v>
       </c>
-      <c r="D24" s="5">
+      <c r="D24" s="3">
         <v>218.4</v>
       </c>
-      <c r="E24" s="5">
+      <c r="E24" s="3">
         <v>218.6</v>
       </c>
-      <c r="F24" s="5">
+      <c r="F24" s="3">
         <v>218.9</v>
       </c>
-      <c r="G24" s="5">
+      <c r="G24" s="3">
         <v>219.5</v>
       </c>
-      <c r="H24" s="5">
+      <c r="H24" s="3">
         <v>220</v>
       </c>
-      <c r="I24" s="5">
+      <c r="I24" s="3">
         <v>220.7</v>
       </c>
-      <c r="J24" s="5">
+      <c r="J24" s="3">
         <v>221.1</v>
       </c>
-      <c r="K24" s="5">
+      <c r="K24" s="3">
         <v>221.2</v>
       </c>
-      <c r="L24" s="5">
+      <c r="L24" s="3">
         <v>221.5</v>
       </c>
-      <c r="M24" s="5">
+      <c r="M24" s="3">
         <v>221.4</v>
       </c>
-      <c r="N24" s="5">
+      <c r="N24" s="3">
         <v>219.7</v>
       </c>
-      <c r="O24" s="2"/>
-    </row>
-    <row r="25" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="3">
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A25" s="1">
         <v>1995</v>
       </c>
-      <c r="B25" s="5">
+      <c r="B25" s="3">
         <v>222.2</v>
       </c>
-      <c r="C25" s="5">
+      <c r="C25" s="3">
         <v>222.9</v>
       </c>
-      <c r="D25" s="5">
+      <c r="D25" s="3">
         <v>223.6</v>
       </c>
-      <c r="E25" s="5">
+      <c r="E25" s="3">
         <v>224.3</v>
       </c>
-      <c r="F25" s="5">
+      <c r="F25" s="3">
         <v>224.7</v>
       </c>
-      <c r="G25" s="5">
+      <c r="G25" s="3">
         <v>225.2</v>
       </c>
-      <c r="H25" s="5">
+      <c r="H25" s="3">
         <v>225.3</v>
       </c>
-      <c r="I25" s="5">
+      <c r="I25" s="3">
         <v>225.7</v>
       </c>
-      <c r="J25" s="5">
+      <c r="J25" s="3">
         <v>226.1</v>
       </c>
-      <c r="K25" s="5">
+      <c r="K25" s="3">
         <v>226.7</v>
       </c>
-      <c r="L25" s="5">
+      <c r="L25" s="3">
         <v>226.5</v>
       </c>
-      <c r="M25" s="5">
+      <c r="M25" s="3">
         <v>226.4</v>
       </c>
-      <c r="N25" s="5">
+      <c r="N25" s="3">
         <v>225</v>
       </c>
-      <c r="O25" s="2"/>
-    </row>
-    <row r="26" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="3">
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A26" s="1">
         <v>1996</v>
       </c>
-      <c r="B26" s="5">
+      <c r="B26" s="3">
         <v>227.5</v>
       </c>
-      <c r="C26" s="5">
+      <c r="C26" s="3">
         <v>228.3</v>
       </c>
-      <c r="D26" s="5">
+      <c r="D26" s="3">
         <v>229.4</v>
       </c>
-      <c r="E26" s="5">
+      <c r="E26" s="3">
         <v>230.2</v>
       </c>
-      <c r="F26" s="5">
+      <c r="F26" s="3">
         <v>230.8</v>
       </c>
-      <c r="G26" s="5">
+      <c r="G26" s="3">
         <v>230.9</v>
       </c>
-      <c r="H26" s="5">
+      <c r="H26" s="3">
         <v>231.3</v>
       </c>
-      <c r="I26" s="5">
+      <c r="I26" s="3">
         <v>231.5</v>
       </c>
-      <c r="J26" s="5">
+      <c r="J26" s="3">
         <v>232.3</v>
       </c>
-      <c r="K26" s="5">
+      <c r="K26" s="3">
         <v>233</v>
       </c>
-      <c r="L26" s="5">
+      <c r="L26" s="3">
         <v>233.4</v>
       </c>
-      <c r="M26" s="5">
+      <c r="M26" s="3">
         <v>233.4</v>
       </c>
-      <c r="N26" s="5">
+      <c r="N26" s="3">
         <v>231</v>
       </c>
-      <c r="O26" s="2"/>
-    </row>
-    <row r="27" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="3">
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A27" s="1">
         <v>1997</v>
       </c>
-      <c r="B27" s="5">
+      <c r="B27" s="3">
         <v>234.1</v>
       </c>
-      <c r="C27" s="5">
+      <c r="C27" s="3">
         <v>234.7</v>
       </c>
-      <c r="D27" s="5">
+      <c r="D27" s="3">
         <v>235.2</v>
       </c>
-      <c r="E27" s="5">
+      <c r="E27" s="3">
         <v>235.5</v>
       </c>
-      <c r="F27" s="5">
+      <c r="F27" s="3">
         <v>235.4</v>
       </c>
-      <c r="G27" s="5">
+      <c r="G27" s="3">
         <v>235.8</v>
       </c>
-      <c r="H27" s="5">
+      <c r="H27" s="3">
         <v>235.9</v>
       </c>
-      <c r="I27" s="5">
+      <c r="I27" s="3">
         <v>236.3</v>
       </c>
-      <c r="J27" s="5">
+      <c r="J27" s="3">
         <v>237.1</v>
       </c>
-      <c r="K27" s="5">
+      <c r="K27" s="3">
         <v>237.5</v>
       </c>
-      <c r="L27" s="5">
+      <c r="L27" s="3">
         <v>237.4</v>
       </c>
-      <c r="M27" s="5">
+      <c r="M27" s="3">
         <v>237</v>
       </c>
-      <c r="N27" s="5">
+      <c r="N27" s="3">
         <v>236</v>
       </c>
-      <c r="O27" s="2"/>
-    </row>
-    <row r="28" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="3">
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A28" s="1">
         <v>1998</v>
       </c>
-      <c r="B28" s="5">
+      <c r="B28" s="3">
         <v>237.4</v>
       </c>
-      <c r="C28" s="5">
+      <c r="C28" s="3">
         <v>237.8</v>
       </c>
-      <c r="D28" s="5">
+      <c r="D28" s="3">
         <v>238.1</v>
       </c>
-      <c r="E28" s="5">
+      <c r="E28" s="3">
         <v>238.6</v>
       </c>
-      <c r="F28" s="5">
+      <c r="F28" s="3">
         <v>239</v>
       </c>
-      <c r="G28" s="5">
+      <c r="G28" s="3">
         <v>239.1</v>
       </c>
-      <c r="H28" s="5">
+      <c r="H28" s="3">
         <v>239.4</v>
       </c>
-      <c r="I28" s="5">
+      <c r="I28" s="3">
         <v>239.7</v>
       </c>
-      <c r="J28" s="5">
+      <c r="J28" s="3">
         <v>240</v>
       </c>
-      <c r="K28" s="5">
+      <c r="K28" s="3">
         <v>240.5</v>
       </c>
-      <c r="L28" s="5">
+      <c r="L28" s="3">
         <v>240.5</v>
       </c>
-      <c r="M28" s="5">
+      <c r="M28" s="3">
         <v>240.3</v>
       </c>
-      <c r="N28" s="5">
+      <c r="N28" s="3">
         <v>239.2</v>
       </c>
-      <c r="O28" s="2"/>
-    </row>
-    <row r="29" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="3">
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A29" s="1">
         <v>1999</v>
       </c>
-      <c r="B29" s="5">
+      <c r="B29" s="3">
         <v>240.9</v>
       </c>
-      <c r="C29" s="5">
+      <c r="C29" s="3">
         <v>241.2</v>
       </c>
-      <c r="D29" s="5">
+      <c r="D29" s="3">
         <v>241.9</v>
       </c>
-      <c r="E29" s="5">
+      <c r="E29" s="3">
         <v>243.6</v>
       </c>
-      <c r="F29" s="5">
+      <c r="F29" s="3">
         <v>243.6</v>
       </c>
-      <c r="G29" s="5">
+      <c r="G29" s="3">
         <v>243.7</v>
       </c>
-      <c r="H29" s="5">
+      <c r="H29" s="3">
         <v>244.4</v>
       </c>
-      <c r="I29" s="5">
+      <c r="I29" s="3">
         <v>245.1</v>
       </c>
-      <c r="J29" s="5">
+      <c r="J29" s="3">
         <v>246.2</v>
       </c>
-      <c r="K29" s="5">
+      <c r="K29" s="3">
         <v>246.7</v>
       </c>
-      <c r="L29" s="5">
+      <c r="L29" s="3">
         <v>246.8</v>
       </c>
-      <c r="M29" s="5">
+      <c r="M29" s="3">
         <v>246.8</v>
       </c>
-      <c r="N29" s="5">
+      <c r="N29" s="3">
         <v>244.2</v>
       </c>
-      <c r="O29" s="2"/>
-    </row>
-    <row r="30" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="3">
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A30" s="1">
         <v>2000</v>
       </c>
-      <c r="B30" s="5">
+      <c r="B30" s="3">
         <v>247.6</v>
       </c>
-      <c r="C30" s="5">
+      <c r="C30" s="3">
         <v>249.1</v>
       </c>
-      <c r="D30" s="5">
+      <c r="D30" s="3">
         <v>251.1</v>
       </c>
-      <c r="E30" s="5">
+      <c r="E30" s="3">
         <v>251.2</v>
       </c>
-      <c r="F30" s="5">
+      <c r="F30" s="3">
         <v>251.4</v>
       </c>
-      <c r="G30" s="5">
+      <c r="G30" s="3">
         <v>252.9</v>
       </c>
-      <c r="H30" s="5">
+      <c r="H30" s="3">
         <v>253.4</v>
       </c>
-      <c r="I30" s="5">
+      <c r="I30" s="3">
         <v>253.4</v>
       </c>
-      <c r="J30" s="5">
+      <c r="J30" s="3">
         <v>254.8</v>
       </c>
-      <c r="K30" s="5">
+      <c r="K30" s="3">
         <v>255.1</v>
       </c>
-      <c r="L30" s="5">
+      <c r="L30" s="3">
         <v>255.3</v>
       </c>
-      <c r="M30" s="5">
+      <c r="M30" s="3">
         <v>255.1</v>
       </c>
-      <c r="N30" s="5">
+      <c r="N30" s="3">
         <v>252.5</v>
       </c>
-      <c r="O30" s="2"/>
-    </row>
-    <row r="31" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="3">
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A31" s="1">
         <v>2001</v>
       </c>
-      <c r="B31" s="5">
+      <c r="B31" s="3">
         <v>256.8</v>
       </c>
-      <c r="C31" s="5">
+      <c r="C31" s="3">
         <v>257.89999999999998</v>
       </c>
-      <c r="D31" s="5">
+      <c r="D31" s="3">
         <v>258.5</v>
       </c>
-      <c r="E31" s="5">
+      <c r="E31" s="3">
         <v>259.5</v>
       </c>
-      <c r="F31" s="5">
+      <c r="F31" s="3">
         <v>260.5</v>
       </c>
-      <c r="G31" s="5">
+      <c r="G31" s="3">
         <v>261.10000000000002</v>
       </c>
-      <c r="H31" s="5">
+      <c r="H31" s="3">
         <v>260.3</v>
       </c>
-      <c r="I31" s="5">
+      <c r="I31" s="3">
         <v>260.39999999999998</v>
       </c>
-      <c r="J31" s="5">
+      <c r="J31" s="3">
         <v>261.39999999999998</v>
       </c>
-      <c r="K31" s="5">
+      <c r="K31" s="3">
         <v>260.60000000000002</v>
       </c>
-      <c r="L31" s="5">
+      <c r="L31" s="3">
         <v>260.10000000000002</v>
       </c>
-      <c r="M31" s="5">
+      <c r="M31" s="3">
         <v>259.10000000000002</v>
       </c>
-      <c r="N31" s="5">
+      <c r="N31" s="3">
         <v>259.7</v>
       </c>
-      <c r="O31" s="2"/>
-    </row>
-    <row r="32" spans="1:15" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="3">
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A32" s="1">
         <v>2002</v>
       </c>
-      <c r="B32" s="5">
+      <c r="B32" s="3">
         <v>259.8</v>
       </c>
-      <c r="C32" s="5">
+      <c r="C32" s="3">
         <v>260.8</v>
       </c>
-      <c r="D32" s="5">
+      <c r="D32" s="3">
         <v>262.2</v>
       </c>
-      <c r="E32" s="5">
+      <c r="E32" s="3">
         <v>263.7</v>
       </c>
-      <c r="F32" s="5">
+      <c r="F32" s="3">
         <v>263.60000000000002</v>
       </c>
-      <c r="G32" s="5">
+      <c r="G32" s="3">
         <v>263.89999999999998</v>
       </c>
-      <c r="H32" s="5">
+      <c r="H32" s="3">
         <v>264.10000000000002</v>
       </c>
-      <c r="I32" s="5">
+      <c r="I32" s="3">
         <v>265</v>
       </c>
-      <c r="J32" s="5">
+      <c r="J32" s="3">
         <v>265.39999999999998</v>
       </c>
-      <c r="K32" s="5">
+      <c r="K32" s="3">
         <v>265.89999999999998</v>
       </c>
-      <c r="L32" s="5">
+      <c r="L32" s="3">
         <v>265.89999999999998</v>
       </c>
-      <c r="M32" s="5">
+      <c r="M32" s="3">
         <v>265.3</v>
       </c>
-      <c r="N32" s="5">
+      <c r="N32" s="3">
         <v>263.8</v>
       </c>
-      <c r="O32" s="1"/>
-    </row>
-    <row r="33" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="3">
+    </row>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A33" s="1">
         <v>2003</v>
       </c>
-      <c r="B33" s="5">
+      <c r="B33" s="3">
         <v>266.39999999999998</v>
       </c>
-      <c r="C33" s="5">
+      <c r="C33" s="3">
         <v>268.60000000000002</v>
       </c>
-      <c r="D33" s="5">
+      <c r="D33" s="3">
         <v>270.2</v>
       </c>
-      <c r="E33" s="5">
+      <c r="E33" s="3">
         <v>269.5</v>
       </c>
-      <c r="F33" s="5">
+      <c r="F33" s="3">
         <v>269.10000000000002</v>
       </c>
-      <c r="G33" s="5">
+      <c r="G33" s="3">
         <v>269.5</v>
       </c>
-      <c r="H33" s="5">
+      <c r="H33" s="3">
         <v>269.7</v>
       </c>
-      <c r="I33" s="5">
+      <c r="I33" s="3">
         <v>270.7</v>
       </c>
-      <c r="J33" s="5">
+      <c r="J33" s="3">
         <v>271.60000000000002</v>
       </c>
-      <c r="K33" s="5">
+      <c r="K33" s="3">
         <v>271.39999999999998</v>
       </c>
-      <c r="L33" s="5">
+      <c r="L33" s="3">
         <v>270.60000000000002</v>
       </c>
-      <c r="M33" s="5">
+      <c r="M33" s="3">
         <v>270.3</v>
       </c>
-      <c r="N33" s="5">
+      <c r="N33" s="3">
         <v>269.8</v>
       </c>
-      <c r="O33" s="2"/>
-    </row>
-    <row r="34" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="3">
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A34" s="1">
         <v>2004</v>
       </c>
-      <c r="B34" s="5">
+      <c r="B34" s="3">
         <v>271.7</v>
       </c>
-      <c r="C34" s="5">
+      <c r="C34" s="3">
         <v>273.2</v>
       </c>
-      <c r="D34" s="5">
+      <c r="D34" s="3">
         <v>274.89999999999998</v>
       </c>
-      <c r="E34" s="5">
+      <c r="E34" s="3">
         <v>275.8</v>
       </c>
-      <c r="F34" s="5">
+      <c r="F34" s="3">
         <v>277.3</v>
       </c>
-      <c r="G34" s="5">
+      <c r="G34" s="3">
         <v>278.2</v>
       </c>
-      <c r="H34" s="5">
+      <c r="H34" s="3">
         <v>277.8</v>
       </c>
-      <c r="I34" s="5">
+      <c r="I34" s="3">
         <v>277.89999999999998</v>
       </c>
-      <c r="J34" s="5">
+      <c r="J34" s="3">
         <v>278.5</v>
       </c>
-      <c r="K34" s="5">
+      <c r="K34" s="3">
         <v>280</v>
       </c>
-      <c r="L34" s="5">
+      <c r="L34" s="3">
         <v>280.2</v>
       </c>
-      <c r="M34" s="5">
+      <c r="M34" s="3">
         <v>279.10000000000002</v>
       </c>
-      <c r="N34" s="5">
+      <c r="N34" s="3">
         <v>277</v>
       </c>
-      <c r="O34" s="2"/>
-    </row>
-    <row r="35" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="3">
+    </row>
+    <row r="35" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A35" s="1">
         <v>2005</v>
       </c>
-      <c r="B35" s="5">
+      <c r="B35" s="3">
         <v>279.60000000000002</v>
       </c>
-      <c r="C35" s="5">
+      <c r="C35" s="3">
         <v>281.3</v>
       </c>
-      <c r="D35" s="5">
+      <c r="D35" s="3">
         <v>283.5</v>
       </c>
-      <c r="E35" s="5">
+      <c r="E35" s="3">
         <v>285.39999999999998</v>
       </c>
-      <c r="F35" s="5">
+      <c r="F35" s="3">
         <v>285.2</v>
       </c>
-      <c r="G35" s="5">
+      <c r="G35" s="3">
         <v>285.2</v>
       </c>
-      <c r="H35" s="5">
+      <c r="H35" s="3">
         <v>286.5</v>
       </c>
-      <c r="I35" s="5">
+      <c r="I35" s="3">
         <v>288</v>
       </c>
-      <c r="J35" s="5">
+      <c r="J35" s="3">
         <v>291.5</v>
       </c>
-      <c r="K35" s="5">
+      <c r="K35" s="3">
         <v>292.2</v>
       </c>
-      <c r="L35" s="5">
+      <c r="L35" s="3">
         <v>289.8</v>
       </c>
-      <c r="M35" s="5">
+      <c r="M35" s="3">
         <v>288.60000000000002</v>
       </c>
-      <c r="N35" s="5">
+      <c r="N35" s="3">
         <v>286.39999999999998</v>
       </c>
-      <c r="O35" s="2"/>
-    </row>
-    <row r="36" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="3">
+    </row>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A36" s="1">
         <v>2006</v>
       </c>
-      <c r="B36" s="5">
+      <c r="B36" s="3">
         <v>290.8</v>
       </c>
-      <c r="C36" s="5">
+      <c r="C36" s="3">
         <v>291.39999999999998</v>
       </c>
-      <c r="D36" s="5">
+      <c r="D36" s="3">
         <v>293.10000000000002</v>
       </c>
-      <c r="E36" s="5">
+      <c r="E36" s="3">
         <v>295.5</v>
       </c>
-      <c r="F36" s="5">
+      <c r="F36" s="3">
         <v>296.89999999999998</v>
       </c>
-      <c r="G36" s="5">
+      <c r="G36" s="3">
         <v>297.60000000000002</v>
       </c>
-      <c r="H36" s="5">
+      <c r="H36" s="3">
         <v>298.39999999999998</v>
       </c>
-      <c r="I36" s="5">
+      <c r="I36" s="3">
         <v>299.10000000000002</v>
       </c>
-      <c r="J36" s="5">
+      <c r="J36" s="3">
         <v>297.60000000000002</v>
       </c>
-      <c r="K36" s="5">
+      <c r="K36" s="3">
         <v>296</v>
       </c>
-      <c r="L36" s="5">
+      <c r="L36" s="3">
         <v>295.60000000000002</v>
       </c>
-      <c r="M36" s="5">
+      <c r="M36" s="3">
         <v>296</v>
       </c>
-      <c r="N36" s="5">
+      <c r="N36" s="3">
         <v>295.7</v>
       </c>
-      <c r="O36" s="2"/>
-    </row>
-    <row r="37" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="3">
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A37" s="1">
         <v>2007</v>
       </c>
-      <c r="B37" s="5">
+      <c r="B37" s="3">
         <v>296.89999999999998</v>
       </c>
-      <c r="C37" s="5">
+      <c r="C37" s="3">
         <v>298.5</v>
       </c>
-      <c r="D37" s="5">
+      <c r="D37" s="3">
         <v>301.2</v>
       </c>
-      <c r="E37" s="5">
+      <c r="E37" s="3">
         <v>303.10000000000002</v>
       </c>
-      <c r="F37" s="5">
+      <c r="F37" s="3">
         <v>305</v>
       </c>
-      <c r="G37" s="5">
+      <c r="G37" s="3">
         <v>305.60000000000002</v>
       </c>
-      <c r="H37" s="5">
+      <c r="H37" s="3">
         <v>305.5</v>
       </c>
-      <c r="I37" s="5">
+      <c r="I37" s="3">
         <v>304.89999999999998</v>
       </c>
-      <c r="J37" s="5">
+      <c r="J37" s="3">
         <v>305.8</v>
       </c>
-      <c r="K37" s="5">
+      <c r="K37" s="3">
         <v>306.39999999999998</v>
       </c>
-      <c r="L37" s="5">
+      <c r="L37" s="3">
         <v>308.3</v>
       </c>
-      <c r="M37" s="5">
+      <c r="M37" s="3">
         <v>308.10000000000002</v>
       </c>
-      <c r="N37" s="5">
+      <c r="N37" s="3">
         <v>304.10000000000002</v>
       </c>
-      <c r="O37" s="2"/>
-    </row>
-    <row r="38" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="3">
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A38" s="1">
         <v>2008</v>
       </c>
-      <c r="B38" s="5">
+      <c r="B38" s="3">
         <v>309.60000000000002</v>
       </c>
-      <c r="C38" s="5">
+      <c r="C38" s="3">
         <v>310.5</v>
       </c>
-      <c r="D38" s="5">
+      <c r="D38" s="3">
         <v>313.2</v>
       </c>
-      <c r="E38" s="5">
+      <c r="E38" s="3">
         <v>315.10000000000002</v>
       </c>
-      <c r="F38" s="5">
+      <c r="F38" s="3">
         <v>317.7</v>
       </c>
-      <c r="G38" s="5">
+      <c r="G38" s="3">
         <v>320.89999999999998</v>
       </c>
-      <c r="H38" s="5">
+      <c r="H38" s="3">
         <v>322.60000000000002</v>
       </c>
-      <c r="I38" s="5">
+      <c r="I38" s="3">
         <v>321.3</v>
       </c>
-      <c r="J38" s="5">
+      <c r="J38" s="3">
         <v>320.89999999999998</v>
       </c>
-      <c r="K38" s="5">
+      <c r="K38" s="3">
         <v>317.60000000000002</v>
       </c>
-      <c r="L38" s="5">
+      <c r="L38" s="3">
         <v>311.60000000000002</v>
       </c>
-      <c r="M38" s="5">
+      <c r="M38" s="3">
         <v>308.3</v>
       </c>
-      <c r="N38" s="5">
+      <c r="N38" s="3">
         <v>315.8</v>
       </c>
-      <c r="O38" s="2"/>
-    </row>
-    <row r="39" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="3">
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A39" s="1">
         <v>2009</v>
       </c>
-      <c r="B39" s="5">
+      <c r="B39" s="3">
         <v>309.7</v>
       </c>
-      <c r="C39" s="5">
+      <c r="C39" s="3">
         <v>311.2</v>
       </c>
-      <c r="D39" s="5">
+      <c r="D39" s="3">
         <v>312</v>
       </c>
-      <c r="E39" s="5">
+      <c r="E39" s="3">
         <v>312.8</v>
       </c>
-      <c r="F39" s="5">
+      <c r="F39" s="3">
         <v>313.7</v>
       </c>
-      <c r="G39" s="5">
+      <c r="G39" s="3">
         <v>316.39999999999998</v>
       </c>
-      <c r="H39" s="5">
+      <c r="H39" s="3">
         <v>315.8</v>
       </c>
-      <c r="I39" s="5">
+      <c r="I39" s="3">
         <v>316.60000000000002</v>
       </c>
-      <c r="J39" s="5">
+      <c r="J39" s="3">
         <v>316.8</v>
       </c>
-      <c r="K39" s="5">
+      <c r="K39" s="3">
         <v>317.10000000000002</v>
       </c>
-      <c r="L39" s="5">
+      <c r="L39" s="3">
         <v>317.3</v>
       </c>
-      <c r="M39" s="5">
+      <c r="M39" s="3">
         <v>316.7</v>
       </c>
-      <c r="N39" s="5">
+      <c r="N39" s="3">
         <v>314.7</v>
       </c>
-      <c r="O39" s="2"/>
-    </row>
-    <row r="40" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="3">
+    </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A40" s="1">
         <v>2010</v>
       </c>
-      <c r="B40" s="5">
+      <c r="B40" s="3">
         <v>317.8</v>
       </c>
-      <c r="C40" s="5">
+      <c r="C40" s="3">
         <v>317.89999999999998</v>
       </c>
-      <c r="D40" s="5">
+      <c r="D40" s="3">
         <v>319.2</v>
       </c>
-      <c r="E40" s="5">
+      <c r="E40" s="3">
         <v>319.8</v>
       </c>
-      <c r="F40" s="5">
+      <c r="F40" s="3">
         <v>320</v>
       </c>
-      <c r="G40" s="5">
+      <c r="G40" s="3">
         <v>319.7</v>
       </c>
-      <c r="H40" s="5">
+      <c r="H40" s="3">
         <v>319.8</v>
       </c>
-      <c r="I40" s="5">
+      <c r="I40" s="3">
         <v>320.2</v>
       </c>
-      <c r="J40" s="5">
+      <c r="J40" s="3">
         <v>320.39999999999998</v>
       </c>
-      <c r="K40" s="5">
+      <c r="K40" s="3">
         <v>320.8</v>
       </c>
-      <c r="L40" s="5">
+      <c r="L40" s="3">
         <v>320.89999999999998</v>
       </c>
-      <c r="M40" s="5">
+      <c r="M40" s="3">
         <v>321.5</v>
       </c>
-      <c r="N40" s="5">
+      <c r="N40" s="3">
         <v>319.8</v>
       </c>
-      <c r="O40" s="2"/>
-    </row>
-    <row r="41" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="3">
+    </row>
+    <row r="41" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A41" s="1">
         <v>2011</v>
       </c>
-      <c r="B41" s="5">
+      <c r="B41" s="3">
         <v>323</v>
       </c>
-      <c r="C41" s="5">
+      <c r="C41" s="3">
         <v>324.60000000000002</v>
       </c>
-      <c r="D41" s="5">
+      <c r="D41" s="3">
         <v>327.8</v>
       </c>
-      <c r="E41" s="5">
+      <c r="E41" s="3">
         <v>329.9</v>
       </c>
-      <c r="F41" s="5">
+      <c r="F41" s="3">
         <v>331.5</v>
       </c>
-      <c r="G41" s="5">
+      <c r="G41" s="3">
         <v>331.1</v>
       </c>
-      <c r="H41" s="5">
+      <c r="H41" s="3">
         <v>331.4</v>
       </c>
-      <c r="I41" s="5">
+      <c r="I41" s="3">
         <v>332.3</v>
       </c>
-      <c r="J41" s="5">
+      <c r="J41" s="3">
         <v>332.8</v>
       </c>
-      <c r="K41" s="5">
+      <c r="K41" s="3">
         <v>332.2</v>
       </c>
-      <c r="L41" s="5">
+      <c r="L41" s="3">
         <v>331.9</v>
       </c>
-      <c r="M41" s="5">
+      <c r="M41" s="3">
         <v>331.1</v>
       </c>
-      <c r="N41" s="5">
+      <c r="N41" s="3">
         <v>330</v>
       </c>
-      <c r="O41" s="2"/>
-    </row>
-    <row r="42" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="3">
+    </row>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A42" s="1">
         <v>2012</v>
       </c>
-      <c r="B42" s="5">
+      <c r="B42" s="3">
         <v>332.6</v>
       </c>
-      <c r="C42" s="5">
+      <c r="C42" s="3">
         <v>334</v>
       </c>
-      <c r="D42" s="5">
+      <c r="D42" s="3">
         <v>336.6</v>
       </c>
-      <c r="E42" s="5">
+      <c r="E42" s="3">
         <v>337.6</v>
       </c>
-      <c r="F42" s="5">
+      <c r="F42" s="3">
         <v>337.2</v>
       </c>
-      <c r="G42" s="5">
+      <c r="G42" s="3">
         <v>336.7</v>
       </c>
-      <c r="H42" s="5">
+      <c r="H42" s="3">
         <v>336.2</v>
       </c>
-      <c r="I42" s="5">
+      <c r="I42" s="3">
         <v>338.1</v>
       </c>
-      <c r="J42" s="5">
+      <c r="J42" s="3">
         <v>339.6</v>
       </c>
-      <c r="K42" s="5">
+      <c r="K42" s="3">
         <v>339.5</v>
       </c>
-      <c r="L42" s="5">
+      <c r="L42" s="3">
         <v>337.9</v>
       </c>
-      <c r="M42" s="5">
+      <c r="M42" s="3">
         <v>337</v>
       </c>
-      <c r="N42" s="5">
+      <c r="N42" s="3">
         <v>336.9</v>
       </c>
-      <c r="O42" s="2"/>
-    </row>
-    <row r="43" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="3">
+    </row>
+    <row r="43" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A43" s="1">
         <v>2013</v>
       </c>
-      <c r="B43" s="5">
+      <c r="B43" s="3">
         <v>338</v>
       </c>
-      <c r="C43" s="5">
+      <c r="C43" s="3">
         <v>340.8</v>
       </c>
-      <c r="D43" s="5">
+      <c r="D43" s="3">
         <v>341.7</v>
       </c>
-      <c r="E43" s="5">
+      <c r="E43" s="3">
         <v>341.3</v>
       </c>
-      <c r="F43" s="5">
+      <c r="F43" s="3">
         <v>341.9</v>
       </c>
-      <c r="G43" s="5">
+      <c r="G43" s="3">
         <v>342.8</v>
       </c>
-      <c r="H43" s="5">
+      <c r="H43" s="3">
         <v>342.9</v>
       </c>
-      <c r="I43" s="5">
+      <c r="I43" s="3">
         <v>343.3</v>
       </c>
-      <c r="J43" s="5">
+      <c r="J43" s="3">
         <v>343.8</v>
       </c>
-      <c r="K43" s="5">
+      <c r="K43" s="3">
         <v>342.9</v>
       </c>
-      <c r="L43" s="5">
+      <c r="L43" s="3">
         <v>342.2</v>
       </c>
-      <c r="M43" s="5">
+      <c r="M43" s="3">
         <v>342.2</v>
       </c>
-      <c r="N43" s="5">
+      <c r="N43" s="3">
         <v>342</v>
       </c>
-      <c r="O43" s="2"/>
-    </row>
-    <row r="44" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="3">
+    </row>
+    <row r="44" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A44" s="1">
         <v>2014</v>
       </c>
-      <c r="B44" s="5">
+      <c r="B44" s="3">
         <v>343.5</v>
       </c>
-      <c r="C44" s="5">
+      <c r="C44" s="3">
         <v>344.8</v>
       </c>
-      <c r="D44" s="5">
+      <c r="D44" s="3">
         <v>347</v>
       </c>
-      <c r="E44" s="5">
+      <c r="E44" s="3">
         <v>348.2</v>
       </c>
-      <c r="F44" s="5">
+      <c r="F44" s="3">
         <v>349.4</v>
       </c>
-      <c r="G44" s="5">
+      <c r="G44" s="3">
         <v>350.1</v>
       </c>
-      <c r="H44" s="5">
+      <c r="H44" s="3">
         <v>349.9</v>
       </c>
-      <c r="I44" s="5">
+      <c r="I44" s="3">
         <v>349.3</v>
       </c>
-      <c r="J44" s="5">
+      <c r="J44" s="3">
         <v>349.6</v>
       </c>
-      <c r="K44" s="5">
+      <c r="K44" s="3">
         <v>348.7</v>
       </c>
-      <c r="L44" s="5">
+      <c r="L44" s="3">
         <v>346.9</v>
       </c>
-      <c r="M44" s="5">
+      <c r="M44" s="3">
         <v>344.9</v>
       </c>
-      <c r="N44" s="5">
+      <c r="N44" s="3">
         <v>347.7</v>
       </c>
-      <c r="O44" s="2"/>
-    </row>
-    <row r="45" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="3">
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A45" s="1">
         <v>2015</v>
       </c>
-      <c r="B45" s="5">
+      <c r="B45" s="3">
         <v>343.4</v>
       </c>
-      <c r="C45" s="5">
+      <c r="C45" s="3">
         <v>344.9</v>
       </c>
-      <c r="D45" s="5">
+      <c r="D45" s="3">
         <v>346.9</v>
       </c>
-      <c r="E45" s="5">
+      <c r="E45" s="3">
         <v>347.7</v>
       </c>
-      <c r="F45" s="5">
+      <c r="F45" s="3">
         <v>349.4</v>
       </c>
-      <c r="G45" s="5">
+      <c r="G45" s="3">
         <v>350.7</v>
       </c>
-      <c r="H45" s="5">
+      <c r="H45" s="3">
         <v>350.7</v>
       </c>
-      <c r="I45" s="5">
+      <c r="I45" s="3">
         <v>350.2</v>
       </c>
-      <c r="J45" s="5">
+      <c r="J45" s="3">
         <v>349.7</v>
       </c>
-      <c r="K45" s="5">
+      <c r="K45" s="3">
         <v>349.5</v>
       </c>
-      <c r="L45" s="5">
+      <c r="L45" s="3">
         <v>348.8</v>
       </c>
-      <c r="M45" s="5">
+      <c r="M45" s="3">
         <v>347.6</v>
       </c>
-      <c r="N45" s="5">
+      <c r="N45" s="3">
         <v>348.3</v>
       </c>
-      <c r="O45" s="2"/>
-    </row>
-    <row r="46" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="3">
+    </row>
+    <row r="46" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A46" s="1">
         <v>2016</v>
       </c>
-      <c r="B46" s="5">
+      <c r="B46" s="3">
         <v>348.2</v>
       </c>
-      <c r="C46" s="5">
+      <c r="C46" s="3">
         <v>348.5</v>
       </c>
-      <c r="D46" s="5">
+      <c r="D46" s="3">
         <v>350</v>
       </c>
-      <c r="E46" s="5">
+      <c r="E46" s="3">
         <v>351.7</v>
       </c>
-      <c r="F46" s="5">
+      <c r="F46" s="3">
         <v>353.1</v>
       </c>
-      <c r="G46" s="5">
+      <c r="G46" s="3">
         <v>354.2</v>
       </c>
-      <c r="H46" s="5">
+      <c r="H46" s="3">
         <v>353.7</v>
       </c>
-      <c r="I46" s="5">
+      <c r="I46" s="3">
         <v>354</v>
       </c>
-      <c r="J46" s="5">
+      <c r="J46" s="3">
         <v>354.8</v>
       </c>
-      <c r="K46" s="5">
+      <c r="K46" s="3">
         <v>355.3</v>
       </c>
-      <c r="L46" s="5">
+      <c r="L46" s="3">
         <v>354.7</v>
       </c>
-      <c r="M46" s="5">
+      <c r="M46" s="3">
         <v>354.9</v>
       </c>
-      <c r="N46" s="5">
+      <c r="N46" s="3">
         <v>352.8</v>
       </c>
-      <c r="O46" s="2"/>
-    </row>
-    <row r="47" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="3">
+    </row>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A47" s="1">
         <v>2017</v>
       </c>
-      <c r="B47" s="5">
+      <c r="B47" s="3">
         <v>356.9</v>
       </c>
-      <c r="C47" s="5">
+      <c r="C47" s="3">
         <v>358</v>
       </c>
-      <c r="D47" s="5">
+      <c r="D47" s="3">
         <v>358.3</v>
       </c>
-      <c r="E47" s="5">
+      <c r="E47" s="3">
         <v>359.4</v>
       </c>
-      <c r="F47" s="5">
+      <c r="F47" s="3">
         <v>359.7</v>
       </c>
-      <c r="G47" s="5">
+      <c r="G47" s="3">
         <v>360</v>
       </c>
-      <c r="H47" s="5">
+      <c r="H47" s="3">
         <v>359.8</v>
       </c>
-      <c r="I47" s="5">
+      <c r="I47" s="3">
         <v>360.9</v>
       </c>
-      <c r="J47" s="5">
+      <c r="J47" s="3">
         <v>362.8</v>
       </c>
-      <c r="K47" s="5">
+      <c r="K47" s="3">
         <v>362.5</v>
       </c>
-      <c r="L47" s="5">
+      <c r="L47" s="3">
         <v>362.6</v>
       </c>
-      <c r="M47" s="5">
+      <c r="M47" s="3">
         <v>362.3</v>
       </c>
-      <c r="N47" s="5">
+      <c r="N47" s="3">
         <v>360.3</v>
       </c>
-      <c r="O47" s="2"/>
-    </row>
-    <row r="48" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="3">
+    </row>
+    <row r="48" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A48" s="1">
         <v>2018</v>
       </c>
-      <c r="B48" s="5">
+      <c r="B48" s="3">
         <v>364.3</v>
       </c>
-      <c r="C48" s="5">
+      <c r="C48" s="3">
         <v>366</v>
       </c>
-      <c r="D48" s="5">
+      <c r="D48" s="3">
         <v>366.7</v>
       </c>
-      <c r="E48" s="5">
+      <c r="E48" s="3">
         <v>368.3</v>
       </c>
-      <c r="F48" s="5">
+      <c r="F48" s="3">
         <v>369.8</v>
       </c>
-      <c r="G48" s="5">
+      <c r="G48" s="3">
         <v>370.3</v>
       </c>
-      <c r="H48" s="5">
+      <c r="H48" s="3">
         <v>370.4</v>
       </c>
-      <c r="I48" s="5">
+      <c r="I48" s="3">
         <v>370.7</v>
       </c>
-      <c r="J48" s="5">
+      <c r="J48" s="3">
         <v>371.1</v>
       </c>
-      <c r="K48" s="5">
+      <c r="K48" s="3">
         <v>371.8</v>
       </c>
-      <c r="L48" s="5">
+      <c r="L48" s="3">
         <v>370.6</v>
       </c>
-      <c r="M48" s="5">
+      <c r="M48" s="3">
         <v>369.3</v>
       </c>
-      <c r="N48" s="5">
+      <c r="N48" s="3">
         <v>369.1</v>
       </c>
-      <c r="O48" s="2"/>
-    </row>
-    <row r="49" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="3">
+    </row>
+    <row r="49" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A49" s="1">
         <v>2019</v>
       </c>
-      <c r="B49" s="5">
-        <v>370</v>
-      </c>
-      <c r="C49" s="5">
-        <v>371.5</v>
-      </c>
-      <c r="D49" s="5">
-        <v>373.6</v>
-      </c>
-      <c r="E49" s="5">
-        <v>375.6</v>
-      </c>
-      <c r="F49" s="5">
-        <v>376.4</v>
-      </c>
-      <c r="G49" s="5">
-        <v>376.5</v>
-      </c>
-      <c r="H49" s="5">
-        <v>377.2</v>
-      </c>
-      <c r="I49" s="5">
-        <v>377.1</v>
-      </c>
-      <c r="J49" s="5">
-        <v>377.5</v>
-      </c>
-      <c r="K49" s="5">
-        <v>378.4</v>
-      </c>
-      <c r="L49" s="5">
-        <v>378.2</v>
-      </c>
-      <c r="M49" s="5">
-        <v>377.8</v>
-      </c>
-      <c r="N49" s="5">
-        <v>375.8</v>
-      </c>
-      <c r="O49" s="2"/>
-    </row>
-    <row r="50" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="3">
+      <c r="B49" s="3">
+        <v>369.95400000000001</v>
+      </c>
+      <c r="C49" s="3">
+        <v>371.54700000000003</v>
+      </c>
+      <c r="D49" s="3">
+        <v>373.57499999999999</v>
+      </c>
+      <c r="E49" s="3">
+        <v>375.59</v>
+      </c>
+      <c r="F49" s="3">
+        <v>376.43</v>
+      </c>
+      <c r="G49" s="3">
+        <v>376.48700000000002</v>
+      </c>
+      <c r="H49" s="3">
+        <v>377.16800000000001</v>
+      </c>
+      <c r="I49" s="3">
+        <v>377.149</v>
+      </c>
+      <c r="J49" s="3">
+        <v>377.517</v>
+      </c>
+      <c r="K49" s="3">
+        <v>378.42599999999999</v>
+      </c>
+      <c r="L49" s="3">
+        <v>378.15699999999998</v>
+      </c>
+      <c r="M49" s="3">
+        <v>377.76</v>
+      </c>
+      <c r="N49" s="3">
+        <v>375.81333333333333</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A50" s="1">
         <v>2020</v>
       </c>
-      <c r="B50" s="5">
-        <v>379.2</v>
-      </c>
-      <c r="C50" s="5">
-        <v>380.2</v>
-      </c>
-      <c r="D50" s="5">
-        <v>379.5</v>
-      </c>
-      <c r="E50" s="5">
-        <v>377.2</v>
-      </c>
-      <c r="F50" s="5">
-        <v>377.2</v>
-      </c>
-      <c r="G50" s="5">
-        <v>379.4</v>
-      </c>
-      <c r="H50" s="5">
-        <v>381.3</v>
-      </c>
-      <c r="I50" s="5">
-        <v>382.6</v>
-      </c>
-      <c r="J50" s="5">
-        <v>383.1</v>
-      </c>
-      <c r="K50" s="5">
-        <v>383.2</v>
-      </c>
-      <c r="L50" s="5">
-        <v>382.9</v>
-      </c>
-      <c r="M50" s="5">
-        <v>383.2</v>
-      </c>
-      <c r="N50" s="5">
-        <v>380.8</v>
-      </c>
-      <c r="O50" s="2"/>
-    </row>
-    <row r="51" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="3">
+      <c r="B50" s="3">
+        <v>379.20699999999999</v>
+      </c>
+      <c r="C50" s="3">
+        <v>380.24400000000003</v>
+      </c>
+      <c r="D50" s="3">
+        <v>379.54700000000003</v>
+      </c>
+      <c r="E50" s="3">
+        <v>377.18099999999998</v>
+      </c>
+      <c r="F50" s="3">
+        <v>377.226</v>
+      </c>
+      <c r="G50" s="3">
+        <v>379.41300000000001</v>
+      </c>
+      <c r="H50" s="3">
+        <v>381.31900000000002</v>
+      </c>
+      <c r="I50" s="3">
+        <v>382.57100000000003</v>
+      </c>
+      <c r="J50" s="3">
+        <v>383.07299999999998</v>
+      </c>
+      <c r="K50" s="3">
+        <v>383.16699999999997</v>
+      </c>
+      <c r="L50" s="3">
+        <v>382.94200000000001</v>
+      </c>
+      <c r="M50" s="3">
+        <v>383.17500000000001</v>
+      </c>
+      <c r="N50" s="3">
+        <v>380.75541666666663</v>
+      </c>
+    </row>
+    <row r="51" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A51" s="1">
         <v>2021</v>
       </c>
-      <c r="B51" s="5">
-        <v>384.9</v>
-      </c>
-      <c r="C51" s="5">
-        <v>387.1</v>
-      </c>
-      <c r="D51" s="5">
-        <v>390</v>
-      </c>
-      <c r="E51" s="5">
-        <v>393.2</v>
-      </c>
-      <c r="F51" s="5">
-        <v>396.7</v>
-      </c>
-      <c r="G51" s="5">
-        <v>400.5</v>
-      </c>
-      <c r="H51" s="5">
-        <v>402.4</v>
-      </c>
-      <c r="I51" s="5">
-        <v>403.1</v>
-      </c>
-      <c r="J51" s="5">
-        <v>404.2</v>
-      </c>
-      <c r="K51" s="5">
-        <v>407.6</v>
-      </c>
-      <c r="L51" s="5">
-        <v>409.5</v>
-      </c>
-      <c r="M51" s="5">
-        <v>410.8</v>
-      </c>
-      <c r="N51" s="5">
-        <v>399.2</v>
-      </c>
-      <c r="O51" s="2"/>
-    </row>
-    <row r="52" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="3">
+      <c r="B51" s="3">
+        <v>384.923</v>
+      </c>
+      <c r="C51" s="3">
+        <v>387.13200000000001</v>
+      </c>
+      <c r="D51" s="3">
+        <v>389.983</v>
+      </c>
+      <c r="E51" s="3">
+        <v>393.24799999999999</v>
+      </c>
+      <c r="F51" s="3">
+        <v>396.74799999999999</v>
+      </c>
+      <c r="G51" s="3">
+        <v>400.512</v>
+      </c>
+      <c r="H51" s="3">
+        <v>402.36799999999999</v>
+      </c>
+      <c r="I51" s="3">
+        <v>403.11500000000001</v>
+      </c>
+      <c r="J51" s="3">
+        <v>404.15800000000002</v>
+      </c>
+      <c r="K51" s="3">
+        <v>407.59500000000003</v>
+      </c>
+      <c r="L51" s="3">
+        <v>409.524</v>
+      </c>
+      <c r="M51" s="3">
+        <v>410.76499999999999</v>
+      </c>
+      <c r="N51" s="3">
+        <v>399.17258333333342</v>
+      </c>
+    </row>
+    <row r="52" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A52" s="1">
         <v>2022</v>
       </c>
-      <c r="B52" s="5">
-        <v>414.3</v>
-      </c>
-      <c r="C52" s="5">
-        <v>418.2</v>
-      </c>
-      <c r="D52" s="5">
-        <v>423.9</v>
-      </c>
-      <c r="E52" s="5">
-        <v>426.3</v>
-      </c>
-      <c r="F52" s="5">
-        <v>431</v>
-      </c>
-      <c r="G52" s="5">
-        <v>436.9</v>
-      </c>
-      <c r="H52" s="5">
-        <v>436.8</v>
-      </c>
-      <c r="I52" s="5">
-        <v>436.7</v>
-      </c>
-      <c r="J52" s="5">
-        <v>437.6</v>
-      </c>
-      <c r="K52" s="5">
-        <v>439.4</v>
-      </c>
-      <c r="L52" s="5">
-        <v>439</v>
-      </c>
-      <c r="M52" s="5">
-        <v>437.6</v>
-      </c>
-      <c r="N52" s="5">
-        <v>431.5</v>
-      </c>
-      <c r="O52" s="2"/>
-    </row>
-    <row r="53" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="3">
+      <c r="B52" s="3">
+        <v>414.25200000000001</v>
+      </c>
+      <c r="C52" s="3">
+        <v>418.166</v>
+      </c>
+      <c r="D52" s="3">
+        <v>423.89400000000001</v>
+      </c>
+      <c r="E52" s="3">
+        <v>426.26499999999999</v>
+      </c>
+      <c r="F52" s="3">
+        <v>430.96199999999999</v>
+      </c>
+      <c r="G52" s="3">
+        <v>436.87299999999999</v>
+      </c>
+      <c r="H52" s="3">
+        <v>436.82900000000001</v>
+      </c>
+      <c r="I52" s="3">
+        <v>436.68200000000002</v>
+      </c>
+      <c r="J52" s="3">
+        <v>437.62200000000001</v>
+      </c>
+      <c r="K52" s="3">
+        <v>439.399</v>
+      </c>
+      <c r="L52" s="3">
+        <v>438.95699999999999</v>
+      </c>
+      <c r="M52" s="3">
+        <v>437.61500000000001</v>
+      </c>
+      <c r="N52" s="3">
+        <v>431.45966666666664</v>
+      </c>
+    </row>
+    <row r="53" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A53" s="1">
         <v>2023</v>
       </c>
-      <c r="B53" s="5">
-        <v>441.1</v>
-      </c>
-      <c r="C53" s="5">
-        <v>443.6</v>
-      </c>
-      <c r="D53" s="5">
-        <v>445</v>
-      </c>
-      <c r="E53" s="5">
-        <v>447.3</v>
-      </c>
-      <c r="F53" s="5">
-        <v>448.4</v>
-      </c>
-      <c r="G53" s="5">
-        <v>449.9</v>
-      </c>
-      <c r="H53" s="5">
-        <v>450.7</v>
-      </c>
-      <c r="I53" s="5">
-        <v>452.7</v>
-      </c>
-      <c r="J53" s="5">
-        <v>453.8</v>
-      </c>
-      <c r="K53" s="5">
-        <v>453.6</v>
-      </c>
-      <c r="L53" s="5">
-        <v>452.7</v>
-      </c>
-      <c r="M53" s="5">
-        <v>452.3</v>
-      </c>
-      <c r="N53" s="5">
-        <v>449.3</v>
-      </c>
-      <c r="O53" s="2"/>
-    </row>
-    <row r="54" spans="1:15" ht="12.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="3">
+      <c r="B53" s="3">
+        <v>441.113</v>
+      </c>
+      <c r="C53" s="3">
+        <v>443.57299999999998</v>
+      </c>
+      <c r="D53" s="3">
+        <v>445.04199999999997</v>
+      </c>
+      <c r="E53" s="3">
+        <v>447.29300000000001</v>
+      </c>
+      <c r="F53" s="3">
+        <v>448.42</v>
+      </c>
+      <c r="G53" s="3">
+        <v>449.86599999999999</v>
+      </c>
+      <c r="H53" s="3">
+        <v>450.72399999999999</v>
+      </c>
+      <c r="I53" s="3">
+        <v>452.69</v>
+      </c>
+      <c r="J53" s="3">
+        <v>453.815</v>
+      </c>
+      <c r="K53" s="3">
+        <v>453.64</v>
+      </c>
+      <c r="L53" s="3">
+        <v>452.726</v>
+      </c>
+      <c r="M53" s="3">
+        <v>452.27499999999998</v>
+      </c>
+      <c r="N53" s="3">
+        <v>449.26474999999999</v>
+      </c>
+    </row>
+    <row r="54" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A54" s="1">
         <v>2024</v>
       </c>
-      <c r="B54" s="5">
-        <v>454.7</v>
-      </c>
-      <c r="C54" s="5">
-        <v>457.6</v>
-      </c>
-      <c r="D54" s="5">
-        <v>460.5</v>
-      </c>
-      <c r="E54" s="5">
-        <v>462.3</v>
-      </c>
-      <c r="F54" s="5">
-        <v>463.1</v>
-      </c>
-      <c r="G54" s="5">
-        <v>463.2</v>
-      </c>
-      <c r="H54" s="5">
-        <v>463.8</v>
-      </c>
-      <c r="I54" s="5">
-        <v>464.1</v>
-      </c>
-      <c r="J54" s="5">
-        <v>464.9</v>
-      </c>
-      <c r="K54" s="5">
-        <v>465.4</v>
-      </c>
-      <c r="L54" s="5">
-        <v>465.2</v>
-      </c>
-      <c r="M54" s="5">
-        <v>465.3</v>
-      </c>
-      <c r="N54" s="5">
-        <v>462.5</v>
-      </c>
-      <c r="O54" s="1"/>
+      <c r="B54" s="3">
+        <v>454.73899999999998</v>
+      </c>
+      <c r="C54" s="3">
+        <v>457.553</v>
+      </c>
+      <c r="D54" s="3">
+        <v>460.51100000000002</v>
+      </c>
+      <c r="E54" s="3">
+        <v>462.30399999999997</v>
+      </c>
+      <c r="F54" s="3">
+        <v>463.072</v>
+      </c>
+      <c r="G54" s="3">
+        <v>463.22800000000001</v>
+      </c>
+      <c r="H54" s="3">
+        <v>463.76499999999999</v>
+      </c>
+      <c r="I54" s="3">
+        <v>464.14299999999997</v>
+      </c>
+      <c r="J54" s="3">
+        <v>464.88799999999998</v>
+      </c>
+      <c r="K54" s="3">
+        <v>465.423</v>
+      </c>
+      <c r="L54" s="3">
+        <v>465.17099999999999</v>
+      </c>
+      <c r="M54" s="3">
+        <v>465.33699999999999</v>
+      </c>
+      <c r="N54" s="3">
+        <v>462.51116666666667</v>
+      </c>
+    </row>
+    <row r="55" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A55" s="1">
+        <v>2025</v>
+      </c>
+      <c r="B55" s="3">
+        <v>468.38299999999998</v>
+      </c>
+      <c r="C55" s="3">
+        <v>470.464</v>
+      </c>
+      <c r="D55" s="3">
+        <v>471.52</v>
+      </c>
+      <c r="E55" s="3">
+        <v>472.98899999999998</v>
+      </c>
+      <c r="F55" s="3">
+        <v>473.97699999999998</v>
+      </c>
+      <c r="G55" s="3">
+        <v>475.59300000000002</v>
+      </c>
+      <c r="H55" s="3">
+        <v>476.31099999999998</v>
+      </c>
+      <c r="I55" s="3">
+        <v>477.68</v>
+      </c>
+      <c r="J55" s="3">
+        <v>478.89499999999998</v>
+      </c>
+      <c r="K55" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="L55" s="3">
+        <v>477.89400000000001</v>
+      </c>
+      <c r="M55" s="3">
+        <v>477.79500000000002</v>
+      </c>
+      <c r="N55" s="3">
+        <v>474.99408333333332</v>
+      </c>
+    </row>
+    <row r="57" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A57" s="5" t="s">
+        <v>20</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>